<commit_message>
Giriş kapısı (24 ay) ile net etkiyi pozitife çekmek: model, CİMER metinleri, ekler, F 3-I 253
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012gVZQXddJGKmSE7re5wowB
</commit_message>
<xml_diff>
--- a/kanun/EKLER_PDF/05b_Mali_Model_Excel.xlsx
+++ b/kanun/EKLER_PDF/05b_Mali_Model_Excel.xlsx
@@ -633,7 +633,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Halen kayıtlı mükellef/sigortalı payı (s)</t>
+          <t>Giriş kapısına rağmen halen kayıtlı payı (s, kapı sızıntısı)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -642,13 +642,13 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.45</v>
+        <v>0.08</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.25</v>
+        <v>0.05</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>0.1</v>
+        <v>0.02</v>
       </c>
       <c r="F10" s="4">
         <f>INDEX(C10:E10,$D$2)</f>
@@ -656,7 +656,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Varsayım; en duyarlı girdi</t>
+          <t>Varsayım; en duyarlı girdi; kırılma %12,6</t>
         </is>
       </c>
     </row>
@@ -5434,7 +5434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C46"/>
+  <dimension ref="A1:C47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -5471,10 +5471,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-6.87027382605839</v>
+        <v>0.1685401876655017</v>
       </c>
       <c r="C4" t="n">
-        <v>-21.15048287104712</v>
+        <v>0.2071101442136524</v>
       </c>
     </row>
     <row r="5">
@@ -5484,10 +5484,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-5.615711960095814</v>
+        <v>3.440481618561076</v>
       </c>
       <c r="C5" t="n">
-        <v>-17.34572053058881</v>
+        <v>10.13312694900861</v>
       </c>
     </row>
     <row r="6">
@@ -5497,10 +5497,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>5.611481737048295</v>
+        <v>12.98159300798363</v>
       </c>
       <c r="C6" t="n">
-        <v>16.7171728071596</v>
+        <v>39.0800078948488</v>
       </c>
     </row>
     <row r="8">
@@ -5513,224 +5513,221 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>P0 Teklif (Orta)</t>
+          <t>G0 Güncel teklif: 24 ay giriş kapısı var (Orta, s=0,05)</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-5.615711960095814</v>
+        <v>3.440481618561076</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>P1 Kayıtlı mükellef girişi kapalı (s=0,02)</t>
+          <t>G1 Önceki taslak: kapı yok (s=0,25)</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4.798910655359609</v>
+        <v>-5.615711960095814</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>P2 Geçiş yapan 4/b primini yarı oranda sürdürür</t>
+          <t>G2 Kapı sızıntısı yüksek (s=0,10)</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>-0.6562469600958107</v>
+        <v>1.176433223896855</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>P3 Götürü gider %20</t>
+          <t>G3 Kapı sızıntısı çok yüksek (s=0,20)</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-4.28547111628818</v>
+        <v>-3.35166356543159</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>P4 (e) bendi yok: düz %10,5</t>
+          <t>G4 Kapı + götürü gider %25</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>-6.184724351735566</v>
+        <v>4.096641034006941</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>P5 90 gün prim hibesi yok</t>
+          <t>G5 Kapı + (e) bendi yok: düz %10,5</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>-5.256294785678648</v>
+        <v>2.871469226921322</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>P6 P1 + P3</t>
+          <t>G6 Kapı + 90 gün prim hibesi yok</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>6.129151499167243</v>
+        <v>3.799898792978242</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>P7 P2 + P3</t>
+          <t>G7 Kapı + donanım KDV mahsubu yok</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.6739938837118215</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+        <v>4.066991453937648</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>G8 Kapı yok + geçenler primi yarı oranda sürdürür (s=0,25)</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>-0.6562469600958107</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Kırılma noktası s* (Orta)</t>
         </is>
       </c>
-      <c r="B18" t="n">
+      <c r="B19" t="n">
         <v>0.1259807437568341</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Monte Carlo (4000 deneme), 4. yıl net (mlr TL)</t>
         </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>P5</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>-19.87961294348348</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P5</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>-14.57809594919718</v>
+        <v>0.4161564399132597</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>P25</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>-8.068488246214164</v>
+        <v>1.049682962427455</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>P50</t>
+          <t>P25</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>-3.18916602550339</v>
+        <v>2.199472967881883</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>P75</t>
+          <t>P50</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>-0.1442039354959099</v>
+        <v>3.691419397158119</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>P90</t>
+          <t>P75</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>2.230643774881467</v>
+        <v>5.732956114161137</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>P95</t>
+          <t>P90</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>3.835773403635827</v>
+        <v>8.469459138717374</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>P95</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>10.78599358742183</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t>P(net&gt;0)</t>
         </is>
       </c>
-      <c r="B28" t="n">
-        <v>0.23775</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+      <c r="B29" t="n">
+        <v>0.9665</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
         <is>
           <t>Tornado (Orta tabanı, 4. yıl net değişimi, mlr TL)</t>
         </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>s_kayitli</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>6.792145183992668</v>
-      </c>
-      <c r="C31" t="n">
-        <v>-9.056193578656883</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>n_toplam</t>
+          <t>s_kayitli</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>3.180406834340467</v>
+        <v>2.264048394664222</v>
       </c>
       <c r="C32" t="n">
-        <v>-5.565711960095814</v>
+        <v>-6.792145183992666</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>prim_odeme</t>
+          <t>n_toplam</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>4.959465000000002</v>
+        <v>-1.994560924892043</v>
       </c>
       <c r="C33" t="n">
-        <v>-2.4797325</v>
+        <v>3.490481618561076</v>
       </c>
     </row>
     <row r="34">
@@ -5740,23 +5737,23 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>-1.626025474818223</v>
+        <v>-2.007667819650359</v>
       </c>
       <c r="C34" t="n">
-        <v>1.819638723973632</v>
+        <v>2.235491621544592</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>marj</t>
+          <t>prim_odeme</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>0.7363950961679153</v>
+        <v>0.991892999999999</v>
       </c>
       <c r="C35" t="n">
-        <v>-0.7691530526988487</v>
+        <v>-0.4959465</v>
       </c>
     </row>
     <row r="36">
@@ -5766,140 +5763,153 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>0.5857025562826633</v>
+        <v>0.5857025562826624</v>
       </c>
       <c r="C36" t="n">
-        <v>-0.5857025562826614</v>
+        <v>-0.5857025562826619</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>u_ucretli</t>
+          <t>sigma</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>0.4880854635688858</v>
+        <v>-0.5049834903819694</v>
       </c>
       <c r="C37" t="n">
-        <v>-0.4880854635688839</v>
+        <v>0.01836165816640997</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>sigma</t>
+          <t>u_ucretli</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>-0.4191478474460964</v>
+        <v>0.4880854635688853</v>
       </c>
       <c r="C38" t="n">
-        <v>0.02389036585517025</v>
+        <v>-0.4880854635688848</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>kdv_donanim_pay</t>
+          <t>marj</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>0.3132549176882858</v>
+        <v>0.3815600417466483</v>
       </c>
       <c r="C39" t="n">
-        <v>-0.3132549176882858</v>
+        <v>-0.3881116330528345</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>r_marj_ucretli</t>
+          <t>kdv_donanim_pay</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>0.2530813514801636</v>
+        <v>0.3132549176882858</v>
       </c>
       <c r="C40" t="n">
-        <v>-0.2892358302630424</v>
+        <v>-0.3132549176882868</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>myo_uygun</t>
+          <t>r_marj_ucretli</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>0.2567265531551189</v>
+        <v>0.2530813514801626</v>
       </c>
       <c r="C41" t="n">
-        <v>-0.2567265531551171</v>
+        <v>-0.2892358302630424</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>kgf_alim</t>
+          <t>myo_uygun</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>0.07592440544404888</v>
+        <v>0.2567265531551189</v>
       </c>
       <c r="C42" t="n">
-        <v>-0.1265406757400808</v>
+        <v>-0.2567265531551171</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>kgf_temerrut</t>
+          <t>kgf_alim</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>0.0632703378700409</v>
+        <v>0.07592440544404888</v>
       </c>
       <c r="C43" t="n">
-        <v>-0.1265406757400808</v>
+        <v>-0.1265406757400813</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>bes_vazgecme</t>
+          <t>kgf_temerrut</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>-0.07361091709504318</v>
+        <v>0.06327033787004041</v>
       </c>
       <c r="C44" t="n">
-        <v>0.07361091709504509</v>
+        <v>-0.1265406757400813</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>phi</t>
+          <t>bes_vazgecme</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>0.03464387011085701</v>
+        <v>-0.07361091709504318</v>
       </c>
       <c r="C45" t="n">
-        <v>-0.06928774022171211</v>
+        <v>0.07361091709504509</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
+          <t>phi</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>0.03464387011085701</v>
+      </c>
+      <c r="C46" t="n">
+        <v>-0.06928774022171354</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
           <t>onlem</t>
         </is>
       </c>
-      <c r="B46" t="n">
-        <v>-0.02078632206651306</v>
-      </c>
-      <c r="C46" t="n">
-        <v>0.02078632206651497</v>
+      <c r="B47" t="n">
+        <v>-0.02078632206651402</v>
+      </c>
+      <c r="C47" t="n">
+        <v>0.02078632206651449</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Giriş kapısı kaldırıldı; sigortalılığın sürekliliği (Madde 1 (p)); model, metinler, ekler yenilendi; F 3-I 255
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012gVZQXddJGKmSE7re5wowB
</commit_message>
<xml_diff>
--- a/kanun/EKLER_PDF/05b_Mali_Model_Excel.xlsx
+++ b/kanun/EKLER_PDF/05b_Mali_Model_Excel.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -633,7 +633,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Giriş kapısına rağmen halen kayıtlı payı (s, kapı sızıntısı)</t>
+          <t>Halen kayıtlı olup rejime geçenlerin payı (s)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -642,13 +642,13 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.08</v>
+        <v>0.3</v>
       </c>
       <c r="D10" s="2" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E10" s="2" t="n">
         <v>0.05</v>
-      </c>
-      <c r="E10" s="2" t="n">
-        <v>0.02</v>
       </c>
       <c r="F10" s="4">
         <f>INDEX(C10:E10,$D$2)</f>
@@ -656,29 +656,29 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Varsayım; en duyarlı girdi; kırılma %12,6</t>
+          <t>Varsayım; prim sürdüğü için sonucu az etkiler</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Ücretli ek gelir payı (u)</t>
+          <t>Halen kayıtlı olanın 4/b primine devamı (1 = prim sürer)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>u_ucretli</t>
+          <t>prim_devam</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>0.15</v>
+        <v>1</v>
       </c>
       <c r="F11" s="4">
         <f>INDEX(C11:E11,$D$2)</f>
@@ -686,29 +686,29 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Varsayım</t>
+          <t>Teklif Madde 1 (p)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Götürü gider oranı</t>
+          <t>Ücretli ek gelir payı (u)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>gider</t>
+          <t>u_ucretli</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>0.3</v>
+        <v>0.15</v>
       </c>
       <c r="F12" s="4">
         <f>INDEX(C12:E12,$D$2)</f>
@@ -716,29 +716,29 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Teklif Madde 1 (a)</t>
+          <t>Varsayım</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>BES aktarım oranı (tevkifatın)</t>
+          <t>Götürü gider oranı</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>bes</t>
+          <t>gider</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.03</v>
+        <v>0.3</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.03</v>
+        <v>0.3</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>0.03</v>
+        <v>0.3</v>
       </c>
       <c r="F13" s="4">
         <f>INDEX(C13:E13,$D$2)</f>
@@ -746,29 +746,29 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Teklif Madde 9</t>
+          <t>Teklif Madde 1 (a)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Devlet katkısı oranı</t>
+          <t>BES aktarım oranı (tevkifatın)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>devlet_katki</t>
+          <t>bes</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.2</v>
+        <v>0.03</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>0.2</v>
+        <v>0.03</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>0.2</v>
+        <v>0.03</v>
       </c>
       <c r="F14" s="4">
         <f>INDEX(C14:E14,$D$2)</f>
@@ -776,29 +776,29 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>4632 Ek 1 + 10811 sayılı Karar (ikincil)</t>
+          <t>Teklif Madde 9</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>BES vazgeçme payı</t>
+          <t>Devlet katkısı oranı</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>bes_vazgecme</t>
+          <t>devlet_katki</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
         <v>0.2</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0.35</v>
+        <v>0.2</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="F15" s="4">
         <f>INDEX(C15:E15,$D$2)</f>
@@ -806,29 +806,29 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Varsayım</t>
+          <t>4632 Ek 1 + 10811 sayılı Karar (ikincil)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>MYÖ prim oranı</t>
+          <t>BES vazgeçme payı</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>myo_oran</t>
+          <t>bes_vazgecme</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.21</v>
+        <v>0.2</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0.21</v>
+        <v>0.35</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>0.21</v>
+        <v>0.5</v>
       </c>
       <c r="F16" s="4">
         <f>INDEX(C16:E16,$D$2)</f>
@@ -836,29 +836,29 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>5510 m.81</t>
+          <t>Varsayım</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Hibe prim süresi (ay)</t>
+          <t>MYÖ prim oranı</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>myo_gun_ay</t>
+          <t>myo_oran</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>3</v>
+        <v>0.21</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>3</v>
+        <v>0.21</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>3</v>
+        <v>0.21</v>
       </c>
       <c r="F17" s="4">
         <f>INDEX(C17:E17,$D$2)</f>
@@ -866,29 +866,29 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Teklif 5510 Ek 25 (90 gün)</t>
+          <t>5510 m.81</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>90 gün primi hak edenlerin payı (çakışmasız)</t>
+          <t>Hibe prim süresi (ay)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>myo_uygun</t>
+          <t>myo_gun_ay</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>0.5</v>
+        <v>3</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>0.35</v>
+        <v>3</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>0.2</v>
+        <v>3</v>
       </c>
       <c r="F18" s="4">
         <f>INDEX(C18:E18,$D$2)</f>
@@ -896,29 +896,29 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Varsayım</t>
+          <t>Teklif 5510 Ek 25 (90 gün)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Donanım alan payı</t>
+          <t>90 gün primi hak edenlerin payı (çakışmasız)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>kdv_donanim_pay</t>
+          <t>myo_uygun</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
         <v>0.5</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>0.4</v>
+        <v>0.35</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="F19" s="4">
         <f>INDEX(C19:E19,$D$2)</f>
@@ -933,22 +933,22 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Yıllık donanım KDV ortalaması (TL)</t>
+          <t>Donanım alan payı</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>kdv_donanim_kdv</t>
+          <t>kdv_donanim_pay</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>5000</v>
+        <v>0.5</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>5000</v>
+        <v>0.4</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>5000</v>
+        <v>0.3</v>
       </c>
       <c r="F20" s="4">
         <f>INDEX(C20:E20,$D$2)</f>
@@ -963,22 +963,22 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>KDV mahsup üst sınırı (tevkifatın oranı)</t>
+          <t>Yıllık donanım KDV ortalaması (TL)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>kdv_mahsup_tavan</t>
+          <t>kdv_donanim_kdv</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>0.5</v>
+        <v>5000</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>0.5</v>
+        <v>5000</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>0.5</v>
+        <v>5000</v>
       </c>
       <c r="F21" s="4">
         <f>INDEX(C21:E21,$D$2)</f>
@@ -986,19 +986,19 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Teklif Madde 3 önerisi</t>
+          <t>Varsayım</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Eski rejimde kâr marjı</t>
+          <t>KDV mahsup üst sınırı (tevkifatın oranı)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>marj</t>
+          <t>kdv_mahsup_tavan</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -1016,29 +1016,29 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Varsayım</t>
+          <t>Teklif Madde 3 önerisi</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Eski 4/b yıllık asgari prim (TL)</t>
+          <t>Eski rejimde kâr marjı</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>prim_eski</t>
+          <t>marj</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>141699</v>
+        <v>0.5</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>141699</v>
+        <v>0.5</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>141699</v>
+        <v>0.5</v>
       </c>
       <c r="F23" s="4">
         <f>INDEX(C23:E23,$D$2)</f>
@@ -1046,29 +1046,29 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>33.030×%35,75×12</t>
+          <t>Varsayım</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Eski prim ödeme oranı</t>
+          <t>Eski 4/b yıllık asgari prim (TL)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>prim_odeme</t>
+          <t>prim_eski</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>0.8</v>
+        <v>141699</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>0.8</v>
+        <v>141699</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>0.8</v>
+        <v>141699</v>
       </c>
       <c r="F24" s="4">
         <f>INDEX(C24:E24,$D$2)</f>
@@ -1076,29 +1076,29 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Varsayım</t>
+          <t>33.030×%35,75×12</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Ücretlinin marjinal oranı</t>
+          <t>Eski prim ödeme oranı</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>r_marj_ucretli</t>
+          <t>prim_odeme</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>0.27</v>
+        <v>0.8</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>0.27</v>
+        <v>0.8</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>0.27</v>
+        <v>0.8</v>
       </c>
       <c r="F25" s="4">
         <f>INDEX(C25:E25,$D$2)</f>
@@ -1113,22 +1113,22 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Ücretlinin eski rejimde uyum oranı</t>
+          <t>Ücretlinin marjinal oranı</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>uyum_ucretli</t>
+          <t>r_marj_ucretli</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>0.5</v>
+        <v>0.27</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>0.5</v>
+        <v>0.27</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>0.5</v>
+        <v>0.27</v>
       </c>
       <c r="F26" s="4">
         <f>INDEX(C26:E26,$D$2)</f>
@@ -1143,22 +1143,22 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Kurumsal alıcı payı</t>
+          <t>Ücretlinin eski rejimde uyum oranı</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>kurumsal_pay</t>
+          <t>uyum_ucretli</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="F27" s="4">
         <f>INDEX(C27:E27,$D$2)</f>
@@ -1173,22 +1173,22 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Kurumlar vergisi oranı</t>
+          <t>Kurumsal alıcı payı</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>kv</t>
+          <t>kurumsal_pay</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>0.25</v>
+        <v>0.7</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>0.25</v>
+        <v>0.7</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>0.25</v>
+        <v>0.7</v>
       </c>
       <c r="F28" s="4">
         <f>INDEX(C28:E28,$D$2)</f>
@@ -1196,29 +1196,29 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Varsayım (kanunda %25)</t>
+          <t>Varsayım</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Sahte fatura payı (kurumsal akışta, φ)</t>
+          <t>Kurumlar vergisi oranı</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>phi</t>
+          <t>kv</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>0.02</v>
+        <v>0.25</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>0.01</v>
+        <v>0.25</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>0.005</v>
+        <v>0.25</v>
       </c>
       <c r="F29" s="4">
         <f>INDEX(C29:E29,$D$2)</f>
@@ -1226,29 +1226,29 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Varsayım</t>
+          <t>Varsayım (kanunda %25)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Önlem etkinliği</t>
+          <t>Sahte fatura payı (kurumsal akışta, φ)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>onlem</t>
+          <t>phi</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>0.3</v>
+        <v>0.02</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>0.5</v>
+        <v>0.01</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>0.7</v>
+        <v>0.005</v>
       </c>
       <c r="F30" s="4">
         <f>INDEX(C30:E30,$D$2)</f>
@@ -1263,22 +1263,22 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>KGF kullanım oranı</t>
+          <t>Önlem etkinliği</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>kgf_alim</t>
+          <t>onlem</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>0.08</v>
+        <v>0.3</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>0.05</v>
+        <v>0.5</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>0.03</v>
+        <v>0.7</v>
       </c>
       <c r="F31" s="4">
         <f>INDEX(C31:E31,$D$2)</f>
@@ -1293,22 +1293,22 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>KGF temerrüt oranı</t>
+          <t>KGF kullanım oranı</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>kgf_temerrut</t>
+          <t>kgf_alim</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
-        <v>0.15</v>
+        <v>0.08</v>
       </c>
       <c r="D32" s="2" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>0.06</v>
+        <v>0.03</v>
       </c>
       <c r="F32" s="4">
         <f>INDEX(C32:E32,$D$2)</f>
@@ -1323,22 +1323,22 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>KGF kurtarma oranı</t>
+          <t>KGF temerrüt oranı</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>kgf_kurtarma</t>
+          <t>kgf_temerrut</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
-        <v>0.3</v>
+        <v>0.15</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>0.3</v>
+        <v>0.06</v>
       </c>
       <c r="F33" s="4">
         <f>INDEX(C33:E33,$D$2)</f>
@@ -1353,22 +1353,22 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Kefalet tutarı (hasılatın payı)</t>
+          <t>KGF kurtarma oranı</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>kgf_pay</t>
+          <t>kgf_kurtarma</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="F34" s="4">
         <f>INDEX(C34:E34,$D$2)</f>
@@ -1376,29 +1376,29 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Teklif Madde 8</t>
+          <t>Varsayım</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>PTT UETS birim gideri (TL)</t>
+          <t>Kefalet tutarı (hasılatın payı)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>ptt_birim</t>
+          <t>kgf_pay</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
-        <v>50</v>
+        <v>0.5</v>
       </c>
       <c r="D35" s="2" t="n">
-        <v>50</v>
+        <v>0.5</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>50</v>
+        <v>0.5</v>
       </c>
       <c r="F35" s="4">
         <f>INDEX(C35:E35,$D$2)</f>
@@ -1406,29 +1406,29 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Varsayım</t>
+          <t>Teklif Madde 8</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>UETS tahsis payı</t>
+          <t>PTT UETS birim gideri (TL)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>ptt_pay</t>
+          <t>ptt_birim</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>0.8</v>
+        <v>50</v>
       </c>
       <c r="D36" s="2" t="n">
-        <v>0.8</v>
+        <v>50</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>0.8</v>
+        <v>50</v>
       </c>
       <c r="F36" s="4">
         <f>INDEX(C36:E36,$D$2)</f>
@@ -1443,22 +1443,22 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Tek seferlik BT gideri (TL)</t>
+          <t>UETS tahsis payı</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>bt_tek</t>
+          <t>ptt_pay</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
-        <v>250000000</v>
+        <v>0.8</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>250000000</v>
+        <v>0.8</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>250000000</v>
+        <v>0.8</v>
       </c>
       <c r="F37" s="4">
         <f>INDEX(C37:E37,$D$2)</f>
@@ -1473,22 +1473,22 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Yıllık BT işletme gideri (TL)</t>
+          <t>Tek seferlik BT gideri (TL)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>bt_yillik</t>
+          <t>bt_tek</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
-        <v>50000000</v>
+        <v>250000000</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>50000000</v>
+        <v>250000000</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>50000000</v>
+        <v>250000000</v>
       </c>
       <c r="F38" s="4">
         <f>INDEX(C38:E38,$D$2)</f>
@@ -1503,22 +1503,22 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>İtiraz oranı</t>
+          <t>Yıllık BT işletme gideri (TL)</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>itiraz_oran</t>
+          <t>bt_yillik</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
-        <v>0.04</v>
+        <v>50000000</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>0.04</v>
+        <v>50000000</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>0.04</v>
+        <v>50000000</v>
       </c>
       <c r="F39" s="4">
         <f>INDEX(C39:E39,$D$2)</f>
@@ -1533,22 +1533,22 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>İtiraz birim gideri (TL)</t>
+          <t>İtiraz oranı</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>itiraz_maliyet</t>
+          <t>itiraz_oran</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
-        <v>2000</v>
+        <v>0.04</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>2000</v>
+        <v>0.04</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>2000</v>
+        <v>0.04</v>
       </c>
       <c r="F40" s="4">
         <f>INDEX(C40:E40,$D$2)</f>
@@ -1563,22 +1563,22 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Denetim gideri (brüt tevkifatın oranı)</t>
+          <t>İtiraz birim gideri (TL)</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>denetim</t>
+          <t>itiraz_maliyet</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
-        <v>0.01</v>
+        <v>2000</v>
       </c>
       <c r="D41" s="2" t="n">
-        <v>0.01</v>
+        <v>2000</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>0.01</v>
+        <v>2000</v>
       </c>
       <c r="F41" s="4">
         <f>INDEX(C41:E41,$D$2)</f>
@@ -1590,72 +1590,86 @@
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="4" t="inlineStr">
-        <is>
-          <t>GVK m.103 tarifesi (2026 parantez içi tutarlar)</t>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Denetim gideri (brüt tevkifatın oranı)</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>denetim</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D42" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E42" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F42" s="4">
+        <f>INDEX(C42:E42,$D$2)</f>
+        <v/>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Varsayım</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
+          <t>GVK m.103 tarifesi (2026 parantez içi tutarlar)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
           <t>Dilim üst sınırı (TL)</t>
         </is>
       </c>
-      <c r="B45" s="4" t="inlineStr">
+      <c r="B46" s="4" t="inlineStr">
         <is>
           <t>Oran</t>
         </is>
       </c>
-      <c r="C45" s="4" t="inlineStr">
+      <c r="C46" s="4" t="inlineStr">
         <is>
           <t>Artış (Δ)</t>
         </is>
       </c>
-      <c r="D45" s="4" t="inlineStr">
+      <c r="D46" s="4" t="inlineStr">
         <is>
           <t>Alt sınır</t>
         </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="n">
-        <v>190000</v>
-      </c>
-      <c r="B46" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="C46">
-        <f>B46</f>
-        <v/>
-      </c>
-      <c r="D46" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>400000</v>
+        <v>190000</v>
       </c>
       <c r="B47" t="n">
-        <v>0.2</v>
+        <v>0.15</v>
       </c>
       <c r="C47">
-        <f>B47-B46</f>
-        <v/>
-      </c>
-      <c r="D47">
-        <f>A46</f>
-        <v/>
+        <f>B47</f>
+        <v/>
+      </c>
+      <c r="D47" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>1000000</v>
+        <v>400000</v>
       </c>
       <c r="B48" t="n">
-        <v>0.27</v>
+        <v>0.2</v>
       </c>
       <c r="C48">
         <f>B48-B47</f>
@@ -1668,10 +1682,10 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>5300000</v>
+        <v>1000000</v>
       </c>
       <c r="B49" t="n">
-        <v>0.35</v>
+        <v>0.27</v>
       </c>
       <c r="C49">
         <f>B49-B48</f>
@@ -1684,10 +1698,10 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>1000000000000</v>
+        <v>5300000</v>
       </c>
       <c r="B50" t="n">
-        <v>0.4</v>
+        <v>0.35</v>
       </c>
       <c r="C50">
         <f>B50-B49</f>
@@ -1695,6 +1709,22 @@
       </c>
       <c r="D50">
         <f>A49</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>1000000000000</v>
+      </c>
+      <c r="B51" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C51">
+        <f>B51-B50</f>
+        <v/>
+      </c>
+      <c r="D51">
+        <f>A50</f>
         <v/>
       </c>
     </row>
@@ -1805,11 +1835,11 @@
         <v/>
       </c>
       <c r="F2">
-        <f>(1-Girdiler!$F$12)*D2</f>
+        <f>(1-Girdiler!$F$13)*D2</f>
         <v/>
       </c>
       <c r="G2">
-        <f>SUMPRODUCT((F2&gt;Girdiler!$D$46:$D$50)*(F2-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F2&gt;Girdiler!$D$47:$D$51)*(F2-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H2">
@@ -1817,27 +1847,27 @@
         <v/>
       </c>
       <c r="I2">
-        <f>Girdiler!$F$13*G2*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G2*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J2">
-        <f>IF(D2&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D2&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K2">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G2,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G2,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L2">
-        <f>SUMPRODUCT((Girdiler!$F$22*D2&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D2-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D2&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D2-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M2">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N2">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D2</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D2</f>
         <v/>
       </c>
     </row>
@@ -1862,11 +1892,11 @@
         <v/>
       </c>
       <c r="F3">
-        <f>(1-Girdiler!$F$12)*D3</f>
+        <f>(1-Girdiler!$F$13)*D3</f>
         <v/>
       </c>
       <c r="G3">
-        <f>SUMPRODUCT((F3&gt;Girdiler!$D$46:$D$50)*(F3-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F3&gt;Girdiler!$D$47:$D$51)*(F3-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H3">
@@ -1874,27 +1904,27 @@
         <v/>
       </c>
       <c r="I3">
-        <f>Girdiler!$F$13*G3*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G3*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J3">
-        <f>IF(D3&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D3&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K3">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G3,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G3,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L3">
-        <f>SUMPRODUCT((Girdiler!$F$22*D3&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D3-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D3&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D3-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M3">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N3">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D3</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D3</f>
         <v/>
       </c>
     </row>
@@ -1919,11 +1949,11 @@
         <v/>
       </c>
       <c r="F4">
-        <f>(1-Girdiler!$F$12)*D4</f>
+        <f>(1-Girdiler!$F$13)*D4</f>
         <v/>
       </c>
       <c r="G4">
-        <f>SUMPRODUCT((F4&gt;Girdiler!$D$46:$D$50)*(F4-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F4&gt;Girdiler!$D$47:$D$51)*(F4-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H4">
@@ -1931,27 +1961,27 @@
         <v/>
       </c>
       <c r="I4">
-        <f>Girdiler!$F$13*G4*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G4*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J4">
-        <f>IF(D4&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D4&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K4">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G4,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G4,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L4">
-        <f>SUMPRODUCT((Girdiler!$F$22*D4&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D4-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D4&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D4-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M4">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N4">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D4</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D4</f>
         <v/>
       </c>
     </row>
@@ -1976,11 +2006,11 @@
         <v/>
       </c>
       <c r="F5">
-        <f>(1-Girdiler!$F$12)*D5</f>
+        <f>(1-Girdiler!$F$13)*D5</f>
         <v/>
       </c>
       <c r="G5">
-        <f>SUMPRODUCT((F5&gt;Girdiler!$D$46:$D$50)*(F5-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F5&gt;Girdiler!$D$47:$D$51)*(F5-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H5">
@@ -1988,27 +2018,27 @@
         <v/>
       </c>
       <c r="I5">
-        <f>Girdiler!$F$13*G5*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G5*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J5">
-        <f>IF(D5&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D5&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K5">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G5,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G5,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L5">
-        <f>SUMPRODUCT((Girdiler!$F$22*D5&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D5-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D5&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D5-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M5">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N5">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D5</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D5</f>
         <v/>
       </c>
     </row>
@@ -2033,11 +2063,11 @@
         <v/>
       </c>
       <c r="F6">
-        <f>(1-Girdiler!$F$12)*D6</f>
+        <f>(1-Girdiler!$F$13)*D6</f>
         <v/>
       </c>
       <c r="G6">
-        <f>SUMPRODUCT((F6&gt;Girdiler!$D$46:$D$50)*(F6-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F6&gt;Girdiler!$D$47:$D$51)*(F6-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H6">
@@ -2045,27 +2075,27 @@
         <v/>
       </c>
       <c r="I6">
-        <f>Girdiler!$F$13*G6*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G6*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J6">
-        <f>IF(D6&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D6&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K6">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G6,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G6,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L6">
-        <f>SUMPRODUCT((Girdiler!$F$22*D6&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D6-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D6&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D6-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M6">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N6">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D6</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D6</f>
         <v/>
       </c>
     </row>
@@ -2090,11 +2120,11 @@
         <v/>
       </c>
       <c r="F7">
-        <f>(1-Girdiler!$F$12)*D7</f>
+        <f>(1-Girdiler!$F$13)*D7</f>
         <v/>
       </c>
       <c r="G7">
-        <f>SUMPRODUCT((F7&gt;Girdiler!$D$46:$D$50)*(F7-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F7&gt;Girdiler!$D$47:$D$51)*(F7-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H7">
@@ -2102,27 +2132,27 @@
         <v/>
       </c>
       <c r="I7">
-        <f>Girdiler!$F$13*G7*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G7*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J7">
-        <f>IF(D7&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D7&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K7">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G7,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G7,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L7">
-        <f>SUMPRODUCT((Girdiler!$F$22*D7&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D7-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D7&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D7-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M7">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N7">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D7</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D7</f>
         <v/>
       </c>
     </row>
@@ -2147,11 +2177,11 @@
         <v/>
       </c>
       <c r="F8">
-        <f>(1-Girdiler!$F$12)*D8</f>
+        <f>(1-Girdiler!$F$13)*D8</f>
         <v/>
       </c>
       <c r="G8">
-        <f>SUMPRODUCT((F8&gt;Girdiler!$D$46:$D$50)*(F8-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F8&gt;Girdiler!$D$47:$D$51)*(F8-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H8">
@@ -2159,27 +2189,27 @@
         <v/>
       </c>
       <c r="I8">
-        <f>Girdiler!$F$13*G8*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G8*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J8">
-        <f>IF(D8&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D8&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K8">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G8,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G8,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L8">
-        <f>SUMPRODUCT((Girdiler!$F$22*D8&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D8-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D8&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D8-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M8">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N8">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D8</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D8</f>
         <v/>
       </c>
     </row>
@@ -2204,11 +2234,11 @@
         <v/>
       </c>
       <c r="F9">
-        <f>(1-Girdiler!$F$12)*D9</f>
+        <f>(1-Girdiler!$F$13)*D9</f>
         <v/>
       </c>
       <c r="G9">
-        <f>SUMPRODUCT((F9&gt;Girdiler!$D$46:$D$50)*(F9-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F9&gt;Girdiler!$D$47:$D$51)*(F9-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H9">
@@ -2216,27 +2246,27 @@
         <v/>
       </c>
       <c r="I9">
-        <f>Girdiler!$F$13*G9*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G9*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J9">
-        <f>IF(D9&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D9&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K9">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G9,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G9,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L9">
-        <f>SUMPRODUCT((Girdiler!$F$22*D9&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D9-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D9&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D9-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M9">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N9">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D9</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D9</f>
         <v/>
       </c>
     </row>
@@ -2261,11 +2291,11 @@
         <v/>
       </c>
       <c r="F10">
-        <f>(1-Girdiler!$F$12)*D10</f>
+        <f>(1-Girdiler!$F$13)*D10</f>
         <v/>
       </c>
       <c r="G10">
-        <f>SUMPRODUCT((F10&gt;Girdiler!$D$46:$D$50)*(F10-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F10&gt;Girdiler!$D$47:$D$51)*(F10-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H10">
@@ -2273,27 +2303,27 @@
         <v/>
       </c>
       <c r="I10">
-        <f>Girdiler!$F$13*G10*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G10*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J10">
-        <f>IF(D10&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D10&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K10">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G10,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G10,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L10">
-        <f>SUMPRODUCT((Girdiler!$F$22*D10&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D10-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D10&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D10-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M10">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N10">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D10</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D10</f>
         <v/>
       </c>
     </row>
@@ -2318,11 +2348,11 @@
         <v/>
       </c>
       <c r="F11">
-        <f>(1-Girdiler!$F$12)*D11</f>
+        <f>(1-Girdiler!$F$13)*D11</f>
         <v/>
       </c>
       <c r="G11">
-        <f>SUMPRODUCT((F11&gt;Girdiler!$D$46:$D$50)*(F11-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F11&gt;Girdiler!$D$47:$D$51)*(F11-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H11">
@@ -2330,27 +2360,27 @@
         <v/>
       </c>
       <c r="I11">
-        <f>Girdiler!$F$13*G11*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G11*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J11">
-        <f>IF(D11&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D11&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K11">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G11,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G11,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L11">
-        <f>SUMPRODUCT((Girdiler!$F$22*D11&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D11-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D11&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D11-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M11">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N11">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D11</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D11</f>
         <v/>
       </c>
     </row>
@@ -2375,11 +2405,11 @@
         <v/>
       </c>
       <c r="F12">
-        <f>(1-Girdiler!$F$12)*D12</f>
+        <f>(1-Girdiler!$F$13)*D12</f>
         <v/>
       </c>
       <c r="G12">
-        <f>SUMPRODUCT((F12&gt;Girdiler!$D$46:$D$50)*(F12-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F12&gt;Girdiler!$D$47:$D$51)*(F12-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H12">
@@ -2387,27 +2417,27 @@
         <v/>
       </c>
       <c r="I12">
-        <f>Girdiler!$F$13*G12*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G12*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J12">
-        <f>IF(D12&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D12&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K12">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G12,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G12,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L12">
-        <f>SUMPRODUCT((Girdiler!$F$22*D12&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D12-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D12&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D12-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M12">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N12">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D12</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D12</f>
         <v/>
       </c>
     </row>
@@ -2432,11 +2462,11 @@
         <v/>
       </c>
       <c r="F13">
-        <f>(1-Girdiler!$F$12)*D13</f>
+        <f>(1-Girdiler!$F$13)*D13</f>
         <v/>
       </c>
       <c r="G13">
-        <f>SUMPRODUCT((F13&gt;Girdiler!$D$46:$D$50)*(F13-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F13&gt;Girdiler!$D$47:$D$51)*(F13-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H13">
@@ -2444,27 +2474,27 @@
         <v/>
       </c>
       <c r="I13">
-        <f>Girdiler!$F$13*G13*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G13*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J13">
-        <f>IF(D13&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D13&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K13">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G13,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G13,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L13">
-        <f>SUMPRODUCT((Girdiler!$F$22*D13&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D13-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D13&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D13-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M13">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N13">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D13</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D13</f>
         <v/>
       </c>
     </row>
@@ -2489,11 +2519,11 @@
         <v/>
       </c>
       <c r="F14">
-        <f>(1-Girdiler!$F$12)*D14</f>
+        <f>(1-Girdiler!$F$13)*D14</f>
         <v/>
       </c>
       <c r="G14">
-        <f>SUMPRODUCT((F14&gt;Girdiler!$D$46:$D$50)*(F14-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F14&gt;Girdiler!$D$47:$D$51)*(F14-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H14">
@@ -2501,27 +2531,27 @@
         <v/>
       </c>
       <c r="I14">
-        <f>Girdiler!$F$13*G14*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G14*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J14">
-        <f>IF(D14&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D14&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K14">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G14,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G14,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L14">
-        <f>SUMPRODUCT((Girdiler!$F$22*D14&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D14-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D14&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D14-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M14">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N14">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D14</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D14</f>
         <v/>
       </c>
     </row>
@@ -2546,11 +2576,11 @@
         <v/>
       </c>
       <c r="F15">
-        <f>(1-Girdiler!$F$12)*D15</f>
+        <f>(1-Girdiler!$F$13)*D15</f>
         <v/>
       </c>
       <c r="G15">
-        <f>SUMPRODUCT((F15&gt;Girdiler!$D$46:$D$50)*(F15-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F15&gt;Girdiler!$D$47:$D$51)*(F15-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H15">
@@ -2558,27 +2588,27 @@
         <v/>
       </c>
       <c r="I15">
-        <f>Girdiler!$F$13*G15*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G15*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J15">
-        <f>IF(D15&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D15&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K15">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G15,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G15,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L15">
-        <f>SUMPRODUCT((Girdiler!$F$22*D15&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D15-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D15&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D15-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M15">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N15">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D15</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D15</f>
         <v/>
       </c>
     </row>
@@ -2603,11 +2633,11 @@
         <v/>
       </c>
       <c r="F16">
-        <f>(1-Girdiler!$F$12)*D16</f>
+        <f>(1-Girdiler!$F$13)*D16</f>
         <v/>
       </c>
       <c r="G16">
-        <f>SUMPRODUCT((F16&gt;Girdiler!$D$46:$D$50)*(F16-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F16&gt;Girdiler!$D$47:$D$51)*(F16-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H16">
@@ -2615,27 +2645,27 @@
         <v/>
       </c>
       <c r="I16">
-        <f>Girdiler!$F$13*G16*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G16*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J16">
-        <f>IF(D16&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D16&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K16">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G16,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G16,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L16">
-        <f>SUMPRODUCT((Girdiler!$F$22*D16&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D16-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D16&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D16-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M16">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N16">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D16</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D16</f>
         <v/>
       </c>
     </row>
@@ -2660,11 +2690,11 @@
         <v/>
       </c>
       <c r="F17">
-        <f>(1-Girdiler!$F$12)*D17</f>
+        <f>(1-Girdiler!$F$13)*D17</f>
         <v/>
       </c>
       <c r="G17">
-        <f>SUMPRODUCT((F17&gt;Girdiler!$D$46:$D$50)*(F17-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F17&gt;Girdiler!$D$47:$D$51)*(F17-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H17">
@@ -2672,27 +2702,27 @@
         <v/>
       </c>
       <c r="I17">
-        <f>Girdiler!$F$13*G17*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G17*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J17">
-        <f>IF(D17&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D17&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K17">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G17,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G17,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L17">
-        <f>SUMPRODUCT((Girdiler!$F$22*D17&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D17-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D17&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D17-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M17">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N17">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D17</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D17</f>
         <v/>
       </c>
     </row>
@@ -2717,11 +2747,11 @@
         <v/>
       </c>
       <c r="F18">
-        <f>(1-Girdiler!$F$12)*D18</f>
+        <f>(1-Girdiler!$F$13)*D18</f>
         <v/>
       </c>
       <c r="G18">
-        <f>SUMPRODUCT((F18&gt;Girdiler!$D$46:$D$50)*(F18-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F18&gt;Girdiler!$D$47:$D$51)*(F18-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H18">
@@ -2729,27 +2759,27 @@
         <v/>
       </c>
       <c r="I18">
-        <f>Girdiler!$F$13*G18*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G18*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J18">
-        <f>IF(D18&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D18&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K18">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G18,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G18,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L18">
-        <f>SUMPRODUCT((Girdiler!$F$22*D18&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D18-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D18&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D18-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M18">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N18">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D18</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D18</f>
         <v/>
       </c>
     </row>
@@ -2774,11 +2804,11 @@
         <v/>
       </c>
       <c r="F19">
-        <f>(1-Girdiler!$F$12)*D19</f>
+        <f>(1-Girdiler!$F$13)*D19</f>
         <v/>
       </c>
       <c r="G19">
-        <f>SUMPRODUCT((F19&gt;Girdiler!$D$46:$D$50)*(F19-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F19&gt;Girdiler!$D$47:$D$51)*(F19-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H19">
@@ -2786,27 +2816,27 @@
         <v/>
       </c>
       <c r="I19">
-        <f>Girdiler!$F$13*G19*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G19*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J19">
-        <f>IF(D19&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D19&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K19">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G19,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G19,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L19">
-        <f>SUMPRODUCT((Girdiler!$F$22*D19&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D19-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D19&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D19-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M19">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N19">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D19</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D19</f>
         <v/>
       </c>
     </row>
@@ -2831,11 +2861,11 @@
         <v/>
       </c>
       <c r="F20">
-        <f>(1-Girdiler!$F$12)*D20</f>
+        <f>(1-Girdiler!$F$13)*D20</f>
         <v/>
       </c>
       <c r="G20">
-        <f>SUMPRODUCT((F20&gt;Girdiler!$D$46:$D$50)*(F20-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F20&gt;Girdiler!$D$47:$D$51)*(F20-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H20">
@@ -2843,27 +2873,27 @@
         <v/>
       </c>
       <c r="I20">
-        <f>Girdiler!$F$13*G20*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G20*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J20">
-        <f>IF(D20&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D20&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K20">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G20,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G20,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L20">
-        <f>SUMPRODUCT((Girdiler!$F$22*D20&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D20-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D20&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D20-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M20">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N20">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D20</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D20</f>
         <v/>
       </c>
     </row>
@@ -2888,11 +2918,11 @@
         <v/>
       </c>
       <c r="F21">
-        <f>(1-Girdiler!$F$12)*D21</f>
+        <f>(1-Girdiler!$F$13)*D21</f>
         <v/>
       </c>
       <c r="G21">
-        <f>SUMPRODUCT((F21&gt;Girdiler!$D$46:$D$50)*(F21-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F21&gt;Girdiler!$D$47:$D$51)*(F21-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H21">
@@ -2900,27 +2930,27 @@
         <v/>
       </c>
       <c r="I21">
-        <f>Girdiler!$F$13*G21*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G21*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J21">
-        <f>IF(D21&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D21&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K21">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G21,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G21,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L21">
-        <f>SUMPRODUCT((Girdiler!$F$22*D21&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D21-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D21&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D21-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M21">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N21">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D21</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D21</f>
         <v/>
       </c>
     </row>
@@ -2945,11 +2975,11 @@
         <v/>
       </c>
       <c r="F22">
-        <f>(1-Girdiler!$F$12)*D22</f>
+        <f>(1-Girdiler!$F$13)*D22</f>
         <v/>
       </c>
       <c r="G22">
-        <f>SUMPRODUCT((F22&gt;Girdiler!$D$46:$D$50)*(F22-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F22&gt;Girdiler!$D$47:$D$51)*(F22-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H22">
@@ -2957,27 +2987,27 @@
         <v/>
       </c>
       <c r="I22">
-        <f>Girdiler!$F$13*G22*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G22*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J22">
-        <f>IF(D22&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D22&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K22">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G22,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G22,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L22">
-        <f>SUMPRODUCT((Girdiler!$F$22*D22&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D22-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D22&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D22-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M22">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N22">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D22</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D22</f>
         <v/>
       </c>
     </row>
@@ -3002,11 +3032,11 @@
         <v/>
       </c>
       <c r="F23">
-        <f>(1-Girdiler!$F$12)*D23</f>
+        <f>(1-Girdiler!$F$13)*D23</f>
         <v/>
       </c>
       <c r="G23">
-        <f>SUMPRODUCT((F23&gt;Girdiler!$D$46:$D$50)*(F23-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F23&gt;Girdiler!$D$47:$D$51)*(F23-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H23">
@@ -3014,27 +3044,27 @@
         <v/>
       </c>
       <c r="I23">
-        <f>Girdiler!$F$13*G23*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G23*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J23">
-        <f>IF(D23&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D23&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K23">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G23,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G23,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L23">
-        <f>SUMPRODUCT((Girdiler!$F$22*D23&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D23-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D23&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D23-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M23">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N23">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D23</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D23</f>
         <v/>
       </c>
     </row>
@@ -3059,11 +3089,11 @@
         <v/>
       </c>
       <c r="F24">
-        <f>(1-Girdiler!$F$12)*D24</f>
+        <f>(1-Girdiler!$F$13)*D24</f>
         <v/>
       </c>
       <c r="G24">
-        <f>SUMPRODUCT((F24&gt;Girdiler!$D$46:$D$50)*(F24-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F24&gt;Girdiler!$D$47:$D$51)*(F24-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H24">
@@ -3071,27 +3101,27 @@
         <v/>
       </c>
       <c r="I24">
-        <f>Girdiler!$F$13*G24*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G24*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J24">
-        <f>IF(D24&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D24&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K24">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G24,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G24,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L24">
-        <f>SUMPRODUCT((Girdiler!$F$22*D24&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D24-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D24&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D24-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M24">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N24">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D24</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D24</f>
         <v/>
       </c>
     </row>
@@ -3116,11 +3146,11 @@
         <v/>
       </c>
       <c r="F25">
-        <f>(1-Girdiler!$F$12)*D25</f>
+        <f>(1-Girdiler!$F$13)*D25</f>
         <v/>
       </c>
       <c r="G25">
-        <f>SUMPRODUCT((F25&gt;Girdiler!$D$46:$D$50)*(F25-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F25&gt;Girdiler!$D$47:$D$51)*(F25-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H25">
@@ -3128,27 +3158,27 @@
         <v/>
       </c>
       <c r="I25">
-        <f>Girdiler!$F$13*G25*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G25*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J25">
-        <f>IF(D25&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D25&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K25">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G25,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G25,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L25">
-        <f>SUMPRODUCT((Girdiler!$F$22*D25&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D25-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D25&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D25-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M25">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N25">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D25</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D25</f>
         <v/>
       </c>
     </row>
@@ -3173,11 +3203,11 @@
         <v/>
       </c>
       <c r="F26">
-        <f>(1-Girdiler!$F$12)*D26</f>
+        <f>(1-Girdiler!$F$13)*D26</f>
         <v/>
       </c>
       <c r="G26">
-        <f>SUMPRODUCT((F26&gt;Girdiler!$D$46:$D$50)*(F26-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F26&gt;Girdiler!$D$47:$D$51)*(F26-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H26">
@@ -3185,27 +3215,27 @@
         <v/>
       </c>
       <c r="I26">
-        <f>Girdiler!$F$13*G26*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G26*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J26">
-        <f>IF(D26&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D26&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K26">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G26,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G26,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L26">
-        <f>SUMPRODUCT((Girdiler!$F$22*D26&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D26-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D26&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D26-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M26">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N26">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D26</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D26</f>
         <v/>
       </c>
     </row>
@@ -3230,11 +3260,11 @@
         <v/>
       </c>
       <c r="F27">
-        <f>(1-Girdiler!$F$12)*D27</f>
+        <f>(1-Girdiler!$F$13)*D27</f>
         <v/>
       </c>
       <c r="G27">
-        <f>SUMPRODUCT((F27&gt;Girdiler!$D$46:$D$50)*(F27-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F27&gt;Girdiler!$D$47:$D$51)*(F27-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H27">
@@ -3242,27 +3272,27 @@
         <v/>
       </c>
       <c r="I27">
-        <f>Girdiler!$F$13*G27*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G27*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J27">
-        <f>IF(D27&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D27&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K27">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G27,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G27,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L27">
-        <f>SUMPRODUCT((Girdiler!$F$22*D27&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D27-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D27&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D27-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M27">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N27">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D27</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D27</f>
         <v/>
       </c>
     </row>
@@ -3287,11 +3317,11 @@
         <v/>
       </c>
       <c r="F28">
-        <f>(1-Girdiler!$F$12)*D28</f>
+        <f>(1-Girdiler!$F$13)*D28</f>
         <v/>
       </c>
       <c r="G28">
-        <f>SUMPRODUCT((F28&gt;Girdiler!$D$46:$D$50)*(F28-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F28&gt;Girdiler!$D$47:$D$51)*(F28-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H28">
@@ -3299,27 +3329,27 @@
         <v/>
       </c>
       <c r="I28">
-        <f>Girdiler!$F$13*G28*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G28*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J28">
-        <f>IF(D28&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D28&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K28">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G28,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G28,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L28">
-        <f>SUMPRODUCT((Girdiler!$F$22*D28&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D28-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D28&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D28-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M28">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N28">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D28</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D28</f>
         <v/>
       </c>
     </row>
@@ -3344,11 +3374,11 @@
         <v/>
       </c>
       <c r="F29">
-        <f>(1-Girdiler!$F$12)*D29</f>
+        <f>(1-Girdiler!$F$13)*D29</f>
         <v/>
       </c>
       <c r="G29">
-        <f>SUMPRODUCT((F29&gt;Girdiler!$D$46:$D$50)*(F29-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F29&gt;Girdiler!$D$47:$D$51)*(F29-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H29">
@@ -3356,27 +3386,27 @@
         <v/>
       </c>
       <c r="I29">
-        <f>Girdiler!$F$13*G29*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G29*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J29">
-        <f>IF(D29&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D29&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K29">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G29,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G29,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L29">
-        <f>SUMPRODUCT((Girdiler!$F$22*D29&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D29-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D29&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D29-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M29">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N29">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D29</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D29</f>
         <v/>
       </c>
     </row>
@@ -3401,11 +3431,11 @@
         <v/>
       </c>
       <c r="F30">
-        <f>(1-Girdiler!$F$12)*D30</f>
+        <f>(1-Girdiler!$F$13)*D30</f>
         <v/>
       </c>
       <c r="G30">
-        <f>SUMPRODUCT((F30&gt;Girdiler!$D$46:$D$50)*(F30-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F30&gt;Girdiler!$D$47:$D$51)*(F30-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H30">
@@ -3413,27 +3443,27 @@
         <v/>
       </c>
       <c r="I30">
-        <f>Girdiler!$F$13*G30*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G30*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J30">
-        <f>IF(D30&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D30&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K30">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G30,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G30,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L30">
-        <f>SUMPRODUCT((Girdiler!$F$22*D30&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D30-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D30&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D30-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M30">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N30">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D30</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D30</f>
         <v/>
       </c>
     </row>
@@ -3458,11 +3488,11 @@
         <v/>
       </c>
       <c r="F31">
-        <f>(1-Girdiler!$F$12)*D31</f>
+        <f>(1-Girdiler!$F$13)*D31</f>
         <v/>
       </c>
       <c r="G31">
-        <f>SUMPRODUCT((F31&gt;Girdiler!$D$46:$D$50)*(F31-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F31&gt;Girdiler!$D$47:$D$51)*(F31-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H31">
@@ -3470,27 +3500,27 @@
         <v/>
       </c>
       <c r="I31">
-        <f>Girdiler!$F$13*G31*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G31*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J31">
-        <f>IF(D31&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D31&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K31">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G31,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G31,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L31">
-        <f>SUMPRODUCT((Girdiler!$F$22*D31&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D31-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D31&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D31-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M31">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N31">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D31</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D31</f>
         <v/>
       </c>
     </row>
@@ -3515,11 +3545,11 @@
         <v/>
       </c>
       <c r="F32">
-        <f>(1-Girdiler!$F$12)*D32</f>
+        <f>(1-Girdiler!$F$13)*D32</f>
         <v/>
       </c>
       <c r="G32">
-        <f>SUMPRODUCT((F32&gt;Girdiler!$D$46:$D$50)*(F32-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F32&gt;Girdiler!$D$47:$D$51)*(F32-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H32">
@@ -3527,27 +3557,27 @@
         <v/>
       </c>
       <c r="I32">
-        <f>Girdiler!$F$13*G32*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G32*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J32">
-        <f>IF(D32&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D32&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K32">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G32,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G32,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L32">
-        <f>SUMPRODUCT((Girdiler!$F$22*D32&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D32-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D32&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D32-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M32">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N32">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D32</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D32</f>
         <v/>
       </c>
     </row>
@@ -3572,11 +3602,11 @@
         <v/>
       </c>
       <c r="F33">
-        <f>(1-Girdiler!$F$12)*D33</f>
+        <f>(1-Girdiler!$F$13)*D33</f>
         <v/>
       </c>
       <c r="G33">
-        <f>SUMPRODUCT((F33&gt;Girdiler!$D$46:$D$50)*(F33-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F33&gt;Girdiler!$D$47:$D$51)*(F33-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H33">
@@ -3584,27 +3614,27 @@
         <v/>
       </c>
       <c r="I33">
-        <f>Girdiler!$F$13*G33*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G33*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J33">
-        <f>IF(D33&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D33&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K33">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G33,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G33,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L33">
-        <f>SUMPRODUCT((Girdiler!$F$22*D33&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D33-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D33&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D33-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M33">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N33">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D33</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D33</f>
         <v/>
       </c>
     </row>
@@ -3629,11 +3659,11 @@
         <v/>
       </c>
       <c r="F34">
-        <f>(1-Girdiler!$F$12)*D34</f>
+        <f>(1-Girdiler!$F$13)*D34</f>
         <v/>
       </c>
       <c r="G34">
-        <f>SUMPRODUCT((F34&gt;Girdiler!$D$46:$D$50)*(F34-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F34&gt;Girdiler!$D$47:$D$51)*(F34-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H34">
@@ -3641,27 +3671,27 @@
         <v/>
       </c>
       <c r="I34">
-        <f>Girdiler!$F$13*G34*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G34*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J34">
-        <f>IF(D34&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D34&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K34">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G34,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G34,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L34">
-        <f>SUMPRODUCT((Girdiler!$F$22*D34&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D34-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D34&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D34-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M34">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N34">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D34</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D34</f>
         <v/>
       </c>
     </row>
@@ -3686,11 +3716,11 @@
         <v/>
       </c>
       <c r="F35">
-        <f>(1-Girdiler!$F$12)*D35</f>
+        <f>(1-Girdiler!$F$13)*D35</f>
         <v/>
       </c>
       <c r="G35">
-        <f>SUMPRODUCT((F35&gt;Girdiler!$D$46:$D$50)*(F35-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F35&gt;Girdiler!$D$47:$D$51)*(F35-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H35">
@@ -3698,27 +3728,27 @@
         <v/>
       </c>
       <c r="I35">
-        <f>Girdiler!$F$13*G35*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G35*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J35">
-        <f>IF(D35&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D35&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K35">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G35,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G35,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L35">
-        <f>SUMPRODUCT((Girdiler!$F$22*D35&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D35-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D35&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D35-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M35">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N35">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D35</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D35</f>
         <v/>
       </c>
     </row>
@@ -3743,11 +3773,11 @@
         <v/>
       </c>
       <c r="F36">
-        <f>(1-Girdiler!$F$12)*D36</f>
+        <f>(1-Girdiler!$F$13)*D36</f>
         <v/>
       </c>
       <c r="G36">
-        <f>SUMPRODUCT((F36&gt;Girdiler!$D$46:$D$50)*(F36-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F36&gt;Girdiler!$D$47:$D$51)*(F36-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H36">
@@ -3755,27 +3785,27 @@
         <v/>
       </c>
       <c r="I36">
-        <f>Girdiler!$F$13*G36*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G36*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J36">
-        <f>IF(D36&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D36&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K36">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G36,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G36,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L36">
-        <f>SUMPRODUCT((Girdiler!$F$22*D36&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D36-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D36&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D36-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M36">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N36">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D36</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D36</f>
         <v/>
       </c>
     </row>
@@ -3800,11 +3830,11 @@
         <v/>
       </c>
       <c r="F37">
-        <f>(1-Girdiler!$F$12)*D37</f>
+        <f>(1-Girdiler!$F$13)*D37</f>
         <v/>
       </c>
       <c r="G37">
-        <f>SUMPRODUCT((F37&gt;Girdiler!$D$46:$D$50)*(F37-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F37&gt;Girdiler!$D$47:$D$51)*(F37-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H37">
@@ -3812,27 +3842,27 @@
         <v/>
       </c>
       <c r="I37">
-        <f>Girdiler!$F$13*G37*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G37*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J37">
-        <f>IF(D37&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D37&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K37">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G37,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G37,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L37">
-        <f>SUMPRODUCT((Girdiler!$F$22*D37&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D37-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D37&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D37-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M37">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N37">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D37</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D37</f>
         <v/>
       </c>
     </row>
@@ -3857,11 +3887,11 @@
         <v/>
       </c>
       <c r="F38">
-        <f>(1-Girdiler!$F$12)*D38</f>
+        <f>(1-Girdiler!$F$13)*D38</f>
         <v/>
       </c>
       <c r="G38">
-        <f>SUMPRODUCT((F38&gt;Girdiler!$D$46:$D$50)*(F38-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F38&gt;Girdiler!$D$47:$D$51)*(F38-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H38">
@@ -3869,27 +3899,27 @@
         <v/>
       </c>
       <c r="I38">
-        <f>Girdiler!$F$13*G38*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G38*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J38">
-        <f>IF(D38&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D38&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K38">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G38,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G38,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L38">
-        <f>SUMPRODUCT((Girdiler!$F$22*D38&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D38-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D38&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D38-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M38">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N38">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D38</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D38</f>
         <v/>
       </c>
     </row>
@@ -3914,11 +3944,11 @@
         <v/>
       </c>
       <c r="F39">
-        <f>(1-Girdiler!$F$12)*D39</f>
+        <f>(1-Girdiler!$F$13)*D39</f>
         <v/>
       </c>
       <c r="G39">
-        <f>SUMPRODUCT((F39&gt;Girdiler!$D$46:$D$50)*(F39-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F39&gt;Girdiler!$D$47:$D$51)*(F39-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H39">
@@ -3926,27 +3956,27 @@
         <v/>
       </c>
       <c r="I39">
-        <f>Girdiler!$F$13*G39*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G39*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J39">
-        <f>IF(D39&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D39&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K39">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G39,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G39,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L39">
-        <f>SUMPRODUCT((Girdiler!$F$22*D39&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D39-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D39&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D39-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M39">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N39">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D39</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D39</f>
         <v/>
       </c>
     </row>
@@ -3971,11 +4001,11 @@
         <v/>
       </c>
       <c r="F40">
-        <f>(1-Girdiler!$F$12)*D40</f>
+        <f>(1-Girdiler!$F$13)*D40</f>
         <v/>
       </c>
       <c r="G40">
-        <f>SUMPRODUCT((F40&gt;Girdiler!$D$46:$D$50)*(F40-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F40&gt;Girdiler!$D$47:$D$51)*(F40-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H40">
@@ -3983,27 +4013,27 @@
         <v/>
       </c>
       <c r="I40">
-        <f>Girdiler!$F$13*G40*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G40*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J40">
-        <f>IF(D40&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D40&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K40">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G40,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G40,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L40">
-        <f>SUMPRODUCT((Girdiler!$F$22*D40&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D40-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D40&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D40-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M40">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N40">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D40</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D40</f>
         <v/>
       </c>
     </row>
@@ -4028,11 +4058,11 @@
         <v/>
       </c>
       <c r="F41">
-        <f>(1-Girdiler!$F$12)*D41</f>
+        <f>(1-Girdiler!$F$13)*D41</f>
         <v/>
       </c>
       <c r="G41">
-        <f>SUMPRODUCT((F41&gt;Girdiler!$D$46:$D$50)*(F41-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F41&gt;Girdiler!$D$47:$D$51)*(F41-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H41">
@@ -4040,27 +4070,27 @@
         <v/>
       </c>
       <c r="I41">
-        <f>Girdiler!$F$13*G41*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G41*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J41">
-        <f>IF(D41&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D41&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K41">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G41,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G41,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L41">
-        <f>SUMPRODUCT((Girdiler!$F$22*D41&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D41-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D41&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D41-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M41">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N41">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D41</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D41</f>
         <v/>
       </c>
     </row>
@@ -4085,11 +4115,11 @@
         <v/>
       </c>
       <c r="F42">
-        <f>(1-Girdiler!$F$12)*D42</f>
+        <f>(1-Girdiler!$F$13)*D42</f>
         <v/>
       </c>
       <c r="G42">
-        <f>SUMPRODUCT((F42&gt;Girdiler!$D$46:$D$50)*(F42-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F42&gt;Girdiler!$D$47:$D$51)*(F42-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H42">
@@ -4097,27 +4127,27 @@
         <v/>
       </c>
       <c r="I42">
-        <f>Girdiler!$F$13*G42*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G42*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J42">
-        <f>IF(D42&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D42&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K42">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G42,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G42,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L42">
-        <f>SUMPRODUCT((Girdiler!$F$22*D42&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D42-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D42&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D42-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M42">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N42">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D42</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D42</f>
         <v/>
       </c>
     </row>
@@ -4142,11 +4172,11 @@
         <v/>
       </c>
       <c r="F43">
-        <f>(1-Girdiler!$F$12)*D43</f>
+        <f>(1-Girdiler!$F$13)*D43</f>
         <v/>
       </c>
       <c r="G43">
-        <f>SUMPRODUCT((F43&gt;Girdiler!$D$46:$D$50)*(F43-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F43&gt;Girdiler!$D$47:$D$51)*(F43-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H43">
@@ -4154,27 +4184,27 @@
         <v/>
       </c>
       <c r="I43">
-        <f>Girdiler!$F$13*G43*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G43*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J43">
-        <f>IF(D43&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D43&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K43">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G43,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G43,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L43">
-        <f>SUMPRODUCT((Girdiler!$F$22*D43&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D43-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D43&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D43-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M43">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N43">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D43</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D43</f>
         <v/>
       </c>
     </row>
@@ -4199,11 +4229,11 @@
         <v/>
       </c>
       <c r="F44">
-        <f>(1-Girdiler!$F$12)*D44</f>
+        <f>(1-Girdiler!$F$13)*D44</f>
         <v/>
       </c>
       <c r="G44">
-        <f>SUMPRODUCT((F44&gt;Girdiler!$D$46:$D$50)*(F44-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F44&gt;Girdiler!$D$47:$D$51)*(F44-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H44">
@@ -4211,27 +4241,27 @@
         <v/>
       </c>
       <c r="I44">
-        <f>Girdiler!$F$13*G44*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G44*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J44">
-        <f>IF(D44&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D44&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K44">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G44,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G44,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L44">
-        <f>SUMPRODUCT((Girdiler!$F$22*D44&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D44-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D44&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D44-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M44">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N44">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D44</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D44</f>
         <v/>
       </c>
     </row>
@@ -4256,11 +4286,11 @@
         <v/>
       </c>
       <c r="F45">
-        <f>(1-Girdiler!$F$12)*D45</f>
+        <f>(1-Girdiler!$F$13)*D45</f>
         <v/>
       </c>
       <c r="G45">
-        <f>SUMPRODUCT((F45&gt;Girdiler!$D$46:$D$50)*(F45-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F45&gt;Girdiler!$D$47:$D$51)*(F45-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H45">
@@ -4268,27 +4298,27 @@
         <v/>
       </c>
       <c r="I45">
-        <f>Girdiler!$F$13*G45*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G45*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J45">
-        <f>IF(D45&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D45&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K45">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G45,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G45,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L45">
-        <f>SUMPRODUCT((Girdiler!$F$22*D45&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D45-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D45&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D45-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M45">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N45">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D45</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D45</f>
         <v/>
       </c>
     </row>
@@ -4313,11 +4343,11 @@
         <v/>
       </c>
       <c r="F46">
-        <f>(1-Girdiler!$F$12)*D46</f>
+        <f>(1-Girdiler!$F$13)*D46</f>
         <v/>
       </c>
       <c r="G46">
-        <f>SUMPRODUCT((F46&gt;Girdiler!$D$46:$D$50)*(F46-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F46&gt;Girdiler!$D$47:$D$51)*(F46-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H46">
@@ -4325,27 +4355,27 @@
         <v/>
       </c>
       <c r="I46">
-        <f>Girdiler!$F$13*G46*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G46*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J46">
-        <f>IF(D46&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D46&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K46">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G46,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G46,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L46">
-        <f>SUMPRODUCT((Girdiler!$F$22*D46&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D46-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D46&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D46-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M46">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N46">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D46</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D46</f>
         <v/>
       </c>
     </row>
@@ -4370,11 +4400,11 @@
         <v/>
       </c>
       <c r="F47">
-        <f>(1-Girdiler!$F$12)*D47</f>
+        <f>(1-Girdiler!$F$13)*D47</f>
         <v/>
       </c>
       <c r="G47">
-        <f>SUMPRODUCT((F47&gt;Girdiler!$D$46:$D$50)*(F47-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F47&gt;Girdiler!$D$47:$D$51)*(F47-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H47">
@@ -4382,27 +4412,27 @@
         <v/>
       </c>
       <c r="I47">
-        <f>Girdiler!$F$13*G47*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G47*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J47">
-        <f>IF(D47&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D47&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K47">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G47,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G47,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L47">
-        <f>SUMPRODUCT((Girdiler!$F$22*D47&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D47-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D47&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D47-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M47">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N47">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D47</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D47</f>
         <v/>
       </c>
     </row>
@@ -4427,11 +4457,11 @@
         <v/>
       </c>
       <c r="F48">
-        <f>(1-Girdiler!$F$12)*D48</f>
+        <f>(1-Girdiler!$F$13)*D48</f>
         <v/>
       </c>
       <c r="G48">
-        <f>SUMPRODUCT((F48&gt;Girdiler!$D$46:$D$50)*(F48-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F48&gt;Girdiler!$D$47:$D$51)*(F48-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H48">
@@ -4439,27 +4469,27 @@
         <v/>
       </c>
       <c r="I48">
-        <f>Girdiler!$F$13*G48*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G48*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J48">
-        <f>IF(D48&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D48&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K48">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G48,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G48,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L48">
-        <f>SUMPRODUCT((Girdiler!$F$22*D48&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D48-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D48&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D48-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M48">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N48">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D48</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D48</f>
         <v/>
       </c>
     </row>
@@ -4484,11 +4514,11 @@
         <v/>
       </c>
       <c r="F49">
-        <f>(1-Girdiler!$F$12)*D49</f>
+        <f>(1-Girdiler!$F$13)*D49</f>
         <v/>
       </c>
       <c r="G49">
-        <f>SUMPRODUCT((F49&gt;Girdiler!$D$46:$D$50)*(F49-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F49&gt;Girdiler!$D$47:$D$51)*(F49-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H49">
@@ -4496,27 +4526,27 @@
         <v/>
       </c>
       <c r="I49">
-        <f>Girdiler!$F$13*G49*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G49*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J49">
-        <f>IF(D49&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D49&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K49">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G49,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G49,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L49">
-        <f>SUMPRODUCT((Girdiler!$F$22*D49&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D49-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D49&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D49-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M49">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N49">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D49</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D49</f>
         <v/>
       </c>
     </row>
@@ -4541,11 +4571,11 @@
         <v/>
       </c>
       <c r="F50">
-        <f>(1-Girdiler!$F$12)*D50</f>
+        <f>(1-Girdiler!$F$13)*D50</f>
         <v/>
       </c>
       <c r="G50">
-        <f>SUMPRODUCT((F50&gt;Girdiler!$D$46:$D$50)*(F50-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F50&gt;Girdiler!$D$47:$D$51)*(F50-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H50">
@@ -4553,27 +4583,27 @@
         <v/>
       </c>
       <c r="I50">
-        <f>Girdiler!$F$13*G50*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G50*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J50">
-        <f>IF(D50&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D50&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K50">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G50,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G50,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L50">
-        <f>SUMPRODUCT((Girdiler!$F$22*D50&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D50-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D50&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D50-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M50">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N50">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D50</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D50</f>
         <v/>
       </c>
     </row>
@@ -4598,11 +4628,11 @@
         <v/>
       </c>
       <c r="F51">
-        <f>(1-Girdiler!$F$12)*D51</f>
+        <f>(1-Girdiler!$F$13)*D51</f>
         <v/>
       </c>
       <c r="G51">
-        <f>SUMPRODUCT((F51&gt;Girdiler!$D$46:$D$50)*(F51-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F51&gt;Girdiler!$D$47:$D$51)*(F51-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H51">
@@ -4610,27 +4640,27 @@
         <v/>
       </c>
       <c r="I51">
-        <f>Girdiler!$F$13*G51*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G51*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J51">
-        <f>IF(D51&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D51&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K51">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G51,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G51,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L51">
-        <f>SUMPRODUCT((Girdiler!$F$22*D51&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D51-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D51&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D51-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M51">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N51">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D51</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D51</f>
         <v/>
       </c>
     </row>
@@ -4655,11 +4685,11 @@
         <v/>
       </c>
       <c r="F52">
-        <f>(1-Girdiler!$F$12)*D52</f>
+        <f>(1-Girdiler!$F$13)*D52</f>
         <v/>
       </c>
       <c r="G52">
-        <f>SUMPRODUCT((F52&gt;Girdiler!$D$46:$D$50)*(F52-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F52&gt;Girdiler!$D$47:$D$51)*(F52-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H52">
@@ -4667,27 +4697,27 @@
         <v/>
       </c>
       <c r="I52">
-        <f>Girdiler!$F$13*G52*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G52*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J52">
-        <f>IF(D52&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D52&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K52">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G52,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G52,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L52">
-        <f>SUMPRODUCT((Girdiler!$F$22*D52&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D52-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D52&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D52-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M52">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N52">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D52</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D52</f>
         <v/>
       </c>
     </row>
@@ -4712,11 +4742,11 @@
         <v/>
       </c>
       <c r="F53">
-        <f>(1-Girdiler!$F$12)*D53</f>
+        <f>(1-Girdiler!$F$13)*D53</f>
         <v/>
       </c>
       <c r="G53">
-        <f>SUMPRODUCT((F53&gt;Girdiler!$D$46:$D$50)*(F53-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F53&gt;Girdiler!$D$47:$D$51)*(F53-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H53">
@@ -4724,27 +4754,27 @@
         <v/>
       </c>
       <c r="I53">
-        <f>Girdiler!$F$13*G53*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G53*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J53">
-        <f>IF(D53&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D53&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K53">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G53,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G53,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L53">
-        <f>SUMPRODUCT((Girdiler!$F$22*D53&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D53-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D53&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D53-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M53">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N53">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D53</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D53</f>
         <v/>
       </c>
     </row>
@@ -4769,11 +4799,11 @@
         <v/>
       </c>
       <c r="F54">
-        <f>(1-Girdiler!$F$12)*D54</f>
+        <f>(1-Girdiler!$F$13)*D54</f>
         <v/>
       </c>
       <c r="G54">
-        <f>SUMPRODUCT((F54&gt;Girdiler!$D$46:$D$50)*(F54-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F54&gt;Girdiler!$D$47:$D$51)*(F54-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H54">
@@ -4781,27 +4811,27 @@
         <v/>
       </c>
       <c r="I54">
-        <f>Girdiler!$F$13*G54*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G54*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J54">
-        <f>IF(D54&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D54&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K54">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G54,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G54,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L54">
-        <f>SUMPRODUCT((Girdiler!$F$22*D54&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D54-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D54&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D54-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M54">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N54">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D54</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D54</f>
         <v/>
       </c>
     </row>
@@ -4826,11 +4856,11 @@
         <v/>
       </c>
       <c r="F55">
-        <f>(1-Girdiler!$F$12)*D55</f>
+        <f>(1-Girdiler!$F$13)*D55</f>
         <v/>
       </c>
       <c r="G55">
-        <f>SUMPRODUCT((F55&gt;Girdiler!$D$46:$D$50)*(F55-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F55&gt;Girdiler!$D$47:$D$51)*(F55-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H55">
@@ -4838,27 +4868,27 @@
         <v/>
       </c>
       <c r="I55">
-        <f>Girdiler!$F$13*G55*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G55*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J55">
-        <f>IF(D55&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D55&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K55">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G55,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G55,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L55">
-        <f>SUMPRODUCT((Girdiler!$F$22*D55&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D55-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D55&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D55-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M55">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N55">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D55</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D55</f>
         <v/>
       </c>
     </row>
@@ -4883,11 +4913,11 @@
         <v/>
       </c>
       <c r="F56">
-        <f>(1-Girdiler!$F$12)*D56</f>
+        <f>(1-Girdiler!$F$13)*D56</f>
         <v/>
       </c>
       <c r="G56">
-        <f>SUMPRODUCT((F56&gt;Girdiler!$D$46:$D$50)*(F56-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F56&gt;Girdiler!$D$47:$D$51)*(F56-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H56">
@@ -4895,27 +4925,27 @@
         <v/>
       </c>
       <c r="I56">
-        <f>Girdiler!$F$13*G56*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G56*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J56">
-        <f>IF(D56&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D56&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K56">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G56,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G56,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L56">
-        <f>SUMPRODUCT((Girdiler!$F$22*D56&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D56-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D56&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D56-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M56">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N56">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D56</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D56</f>
         <v/>
       </c>
     </row>
@@ -4940,11 +4970,11 @@
         <v/>
       </c>
       <c r="F57">
-        <f>(1-Girdiler!$F$12)*D57</f>
+        <f>(1-Girdiler!$F$13)*D57</f>
         <v/>
       </c>
       <c r="G57">
-        <f>SUMPRODUCT((F57&gt;Girdiler!$D$46:$D$50)*(F57-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F57&gt;Girdiler!$D$47:$D$51)*(F57-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H57">
@@ -4952,27 +4982,27 @@
         <v/>
       </c>
       <c r="I57">
-        <f>Girdiler!$F$13*G57*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G57*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J57">
-        <f>IF(D57&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D57&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K57">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G57,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G57,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L57">
-        <f>SUMPRODUCT((Girdiler!$F$22*D57&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D57-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D57&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D57-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M57">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N57">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D57</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D57</f>
         <v/>
       </c>
     </row>
@@ -4997,11 +5027,11 @@
         <v/>
       </c>
       <c r="F58">
-        <f>(1-Girdiler!$F$12)*D58</f>
+        <f>(1-Girdiler!$F$13)*D58</f>
         <v/>
       </c>
       <c r="G58">
-        <f>SUMPRODUCT((F58&gt;Girdiler!$D$46:$D$50)*(F58-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F58&gt;Girdiler!$D$47:$D$51)*(F58-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H58">
@@ -5009,27 +5039,27 @@
         <v/>
       </c>
       <c r="I58">
-        <f>Girdiler!$F$13*G58*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G58*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J58">
-        <f>IF(D58&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D58&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K58">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G58,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G58,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L58">
-        <f>SUMPRODUCT((Girdiler!$F$22*D58&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D58-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D58&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D58-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M58">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N58">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D58</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D58</f>
         <v/>
       </c>
     </row>
@@ -5054,11 +5084,11 @@
         <v/>
       </c>
       <c r="F59">
-        <f>(1-Girdiler!$F$12)*D59</f>
+        <f>(1-Girdiler!$F$13)*D59</f>
         <v/>
       </c>
       <c r="G59">
-        <f>SUMPRODUCT((F59&gt;Girdiler!$D$46:$D$50)*(F59-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F59&gt;Girdiler!$D$47:$D$51)*(F59-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H59">
@@ -5066,27 +5096,27 @@
         <v/>
       </c>
       <c r="I59">
-        <f>Girdiler!$F$13*G59*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G59*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J59">
-        <f>IF(D59&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D59&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K59">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G59,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G59,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L59">
-        <f>SUMPRODUCT((Girdiler!$F$22*D59&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D59-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D59&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D59-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M59">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N59">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D59</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D59</f>
         <v/>
       </c>
     </row>
@@ -5111,11 +5141,11 @@
         <v/>
       </c>
       <c r="F60">
-        <f>(1-Girdiler!$F$12)*D60</f>
+        <f>(1-Girdiler!$F$13)*D60</f>
         <v/>
       </c>
       <c r="G60">
-        <f>SUMPRODUCT((F60&gt;Girdiler!$D$46:$D$50)*(F60-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F60&gt;Girdiler!$D$47:$D$51)*(F60-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H60">
@@ -5123,27 +5153,27 @@
         <v/>
       </c>
       <c r="I60">
-        <f>Girdiler!$F$13*G60*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G60*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J60">
-        <f>IF(D60&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D60&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K60">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G60,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G60,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L60">
-        <f>SUMPRODUCT((Girdiler!$F$22*D60&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D60-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D60&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D60-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M60">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N60">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D60</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D60</f>
         <v/>
       </c>
     </row>
@@ -5168,11 +5198,11 @@
         <v/>
       </c>
       <c r="F61">
-        <f>(1-Girdiler!$F$12)*D61</f>
+        <f>(1-Girdiler!$F$13)*D61</f>
         <v/>
       </c>
       <c r="G61">
-        <f>SUMPRODUCT((F61&gt;Girdiler!$D$46:$D$50)*(F61-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((F61&gt;Girdiler!$D$47:$D$51)*(F61-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="H61">
@@ -5180,27 +5210,27 @@
         <v/>
       </c>
       <c r="I61">
-        <f>Girdiler!$F$13*G61*(1-Girdiler!$F$15)*(1+Girdiler!$F$14)</f>
+        <f>Girdiler!$F$14*G61*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
         <v/>
       </c>
       <c r="J61">
-        <f>IF(D61&gt;=12*Girdiler!$F$6,Girdiler!$F$18*Girdiler!$F$17*Girdiler!$F$6*Girdiler!$F$16,0)</f>
+        <f>IF(D61&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
         <v/>
       </c>
       <c r="K61">
-        <f>Girdiler!$F$19*MIN(Girdiler!$F$21*G61,Girdiler!$F$20)</f>
+        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G61,Girdiler!$F$21)</f>
         <v/>
       </c>
       <c r="L61">
-        <f>SUMPRODUCT((Girdiler!$F$22*D61&gt;Girdiler!$D$46:$D$50)*(Girdiler!$F$22*D61-Girdiler!$D$46:$D$50)*Girdiler!$C$46:$C$50)</f>
+        <f>SUMPRODUCT((Girdiler!$F$23*D61&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D61-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
         <v/>
       </c>
       <c r="M61">
-        <f>Girdiler!$F$24*Girdiler!$F$23</f>
+        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
         <v/>
       </c>
       <c r="N61">
-        <f>Girdiler!$F$26*Girdiler!$F$25*Girdiler!$F$22*D61</f>
+        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D61</f>
         <v/>
       </c>
     </row>
@@ -5324,7 +5354,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>B5*(Girdiler!$F$10*SUMPRODUCT(Hesap!$E$2:$E$61,Hesap!$L$2:$L$61)+Girdiler!$F$11*SUMPRODUCT(Hesap!$E$2:$E$61,Hesap!$N$2:$N$61))</f>
+        <f>B5*(Girdiler!$F$10*SUMPRODUCT(Hesap!$E$2:$E$61,Hesap!$L$2:$L$61)+Girdiler!$F$12*SUMPRODUCT(Hesap!$E$2:$E$61,Hesap!$N$2:$N$61))</f>
         <v/>
       </c>
     </row>
@@ -5346,7 +5376,7 @@
         </is>
       </c>
       <c r="B12">
-        <f>MAX(Girdiler!$F$29*(1-Girdiler!$F$30)*Girdiler!$F$27*B5*B2*(Girdiler!$F$28-B4),0)</f>
+        <f>MAX(Girdiler!$F$30*(1-Girdiler!$F$31)*Girdiler!$F$28*B5*B2*(Girdiler!$F$29-B4),0)</f>
         <v/>
       </c>
     </row>
@@ -5357,7 +5387,7 @@
         </is>
       </c>
       <c r="B13">
-        <f>B5*Girdiler!$F$31*Girdiler!$F$34*B2*Girdiler!$F$32*(1-Girdiler!$F$33)</f>
+        <f>B5*Girdiler!$F$32*Girdiler!$F$35*B2*Girdiler!$F$33*(1-Girdiler!$F$34)</f>
         <v/>
       </c>
     </row>
@@ -5368,7 +5398,7 @@
         </is>
       </c>
       <c r="B14">
-        <f>Girdiler!$F$38</f>
+        <f>Girdiler!$F$39</f>
         <v/>
       </c>
     </row>
@@ -5379,7 +5409,7 @@
         </is>
       </c>
       <c r="B15">
-        <f>B5*Girdiler!$F$39*Girdiler!$F$40</f>
+        <f>B5*Girdiler!$F$40*Girdiler!$F$41</f>
         <v/>
       </c>
     </row>
@@ -5390,7 +5420,7 @@
         </is>
       </c>
       <c r="B16">
-        <f>Girdiler!$F$41*B6</f>
+        <f>Girdiler!$F$42*B6</f>
         <v/>
       </c>
     </row>
@@ -5419,7 +5449,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Not: kırılma noktası s* (net=0 için yutulma payı) Python modelinde ikili aramayla hesaplanmıştır (Senaryolar_Python sayfası).</t>
+          <t>Not: prim sürekliliği (prim_devam=1) ile kırılma noktası yoktur; s=1 için Python varyantı Senaryolar_Python sayfasındadır.</t>
         </is>
       </c>
     </row>
@@ -5471,10 +5501,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.1685401876655017</v>
+        <v>1.084463422748595</v>
       </c>
       <c r="C4" t="n">
-        <v>0.2071101442136524</v>
+        <v>2.986259536424468</v>
       </c>
     </row>
     <row r="5">
@@ -5484,10 +5514,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3.440481618561076</v>
+        <v>4.863742829232634</v>
       </c>
       <c r="C5" t="n">
-        <v>10.13312694900861</v>
+        <v>14.45167175395206</v>
       </c>
     </row>
     <row r="6">
@@ -5497,10 +5527,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>12.98159300798363</v>
+        <v>14.18537328138288</v>
       </c>
       <c r="C6" t="n">
-        <v>39.0800078948488</v>
+        <v>42.73259043346012</v>
       </c>
     </row>
     <row r="8">
@@ -5513,91 +5543,91 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>G0 Güncel teklif: 24 ay giriş kapısı var (Orta, s=0,05)</t>
+          <t>G0 Seçilen: kapısız, halen kayıtlı olanın 4/b primi sürer (s=0,15)</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>3.440481618561076</v>
+        <v>4.863742829232634</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>G1 Önceki taslak: kapı yok (s=0,25)</t>
+          <t>G1 Prim sürekliliği olmasaydı (kapısız, s=0,15)</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-5.615711960095814</v>
+        <v>-1.087615170767367</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>G2 Kapı sızıntısı yüksek (s=0,10)</t>
+          <t>G2 Önceki karar: 24 ay giriş kapısı (s=0,05, prim sürekliliği yok)</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1.176433223896855</v>
+        <v>3.440481618561076</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>G3 Kapı sızıntısı çok yüksek (s=0,20)</t>
+          <t>G3 Harici öneri: düz %15 (%5 prim payı), hibe yok, kapısız (s=0,15)</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-3.35166356543159</v>
+        <v>1.823954910190622</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>G4 Kapı + götürü gider %25</t>
+          <t>G4 Seçilen, herkes geçse (s=1,00)</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>4.096641034006941</v>
+        <v>1.075453047078635</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>G5 Kapı + (e) bendi yok: düz %10,5</t>
+          <t>G5 Seçilen + 90 gün prim hibesi yok</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>2.871469226921322</v>
+        <v>5.2231600036498</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>G6 Kapı + 90 gün prim hibesi yok</t>
+          <t>G6 Seçilen + donanım KDV mahsubu yok</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>3.799898792978242</v>
+        <v>5.490252664609205</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>G7 Kapı + donanım KDV mahsubu yok</t>
+          <t>G7 Seçilen + (e) bendi yok: düz %10,5</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>4.066991453937648</v>
+        <v>4.29473043759288</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>G8 Kapı yok + geçenler primi yarı oranda sürdürür (s=0,25)</t>
+          <t>G8 Seçilen + götürü gider %25</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>-0.6562469600958107</v>
+        <v>5.519902244678498</v>
       </c>
     </row>
     <row r="19">
@@ -5606,8 +5636,10 @@
           <t>Kırılma noktası s* (Orta)</t>
         </is>
       </c>
-      <c r="B19" t="n">
-        <v>0.1259807437568341</v>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>yok</t>
+        </is>
       </c>
     </row>
     <row r="21">
@@ -5624,7 +5656,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.4161564399132597</v>
+        <v>1.371685259209676</v>
       </c>
     </row>
     <row r="23">
@@ -5634,7 +5666,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1.049682962427455</v>
+        <v>1.816043653111378</v>
       </c>
     </row>
     <row r="24">
@@ -5644,7 +5676,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>2.199472967881883</v>
+        <v>2.740448089415021</v>
       </c>
     </row>
     <row r="25">
@@ -5654,7 +5686,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>3.691419397158119</v>
+        <v>4.210833232420195</v>
       </c>
     </row>
     <row r="26">
@@ -5664,7 +5696,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>5.732956114161137</v>
+        <v>6.348701487779011</v>
       </c>
     </row>
     <row r="27">
@@ -5674,7 +5706,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>8.469459138717374</v>
+        <v>9.050144277377949</v>
       </c>
     </row>
     <row r="28">
@@ -5684,7 +5716,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>10.78599358742183</v>
+        <v>11.31276202009183</v>
       </c>
     </row>
     <row r="29">
@@ -5694,7 +5726,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>0.9665</v>
+        <v>0.99875</v>
       </c>
     </row>
     <row r="31">
@@ -5707,209 +5739,209 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>s_kayitli</t>
+          <t>n_toplam</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>2.264048394664222</v>
+        <v>-2.807853045275791</v>
       </c>
       <c r="C32" t="n">
-        <v>-6.792145183992666</v>
+        <v>4.913742829232634</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>n_toplam</t>
+          <t>medyan_W</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>-1.994560924892043</v>
+        <v>-1.816846647234291</v>
       </c>
       <c r="C33" t="n">
-        <v>3.490481618561076</v>
+        <v>2.027565172759112</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>medyan_W</t>
+          <t>s_kayitli</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>-2.007667819650359</v>
+        <v>0.8407871839926644</v>
       </c>
       <c r="C34" t="n">
-        <v>2.235491621544592</v>
+        <v>-0.2802623946642227</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>prim_odeme</t>
+          <t>uyum_ucretli</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>0.991892999999999</v>
+        <v>0.5857025562826614</v>
       </c>
       <c r="C35" t="n">
-        <v>-0.4959465</v>
+        <v>-0.5857025562826629</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>uyum_ucretli</t>
+          <t>marj</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>0.5857025562826624</v>
+        <v>0.5589775689572811</v>
       </c>
       <c r="C36" t="n">
-        <v>-0.5857025562826619</v>
+        <v>-0.5786323428758425</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>sigma</t>
+          <t>u_ucretli</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>-0.5049834903819694</v>
+        <v>0.4880854635688839</v>
       </c>
       <c r="C37" t="n">
-        <v>0.01836165816640997</v>
+        <v>-0.4880854635688858</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>u_ucretli</t>
+          <t>sigma</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>0.4880854635688853</v>
+        <v>-0.4620656689140339</v>
       </c>
       <c r="C38" t="n">
-        <v>-0.4880854635688848</v>
+        <v>0.02112601201078796</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>marj</t>
+          <t>kdv_donanim_pay</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>0.3815600417466483</v>
+        <v>0.3132549176882858</v>
       </c>
       <c r="C39" t="n">
-        <v>-0.3881116330528345</v>
+        <v>-0.3132549176882877</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>kdv_donanim_pay</t>
+          <t>r_marj_ucretli</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>0.3132549176882858</v>
+        <v>0.2530813514801616</v>
       </c>
       <c r="C40" t="n">
-        <v>-0.3132549176882868</v>
+        <v>-0.2892358302630443</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>r_marj_ucretli</t>
+          <t>myo_uygun</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>0.2530813514801626</v>
+        <v>0.2567265531551189</v>
       </c>
       <c r="C41" t="n">
-        <v>-0.2892358302630424</v>
+        <v>-0.2567265531551171</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>myo_uygun</t>
+          <t>kgf_alim</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>0.2567265531551189</v>
+        <v>0.07592440544404792</v>
       </c>
       <c r="C42" t="n">
-        <v>-0.2567265531551171</v>
+        <v>-0.1265406757400818</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>kgf_alim</t>
+          <t>kgf_temerrut</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>0.07592440544404888</v>
+        <v>0.06327033787003994</v>
       </c>
       <c r="C43" t="n">
-        <v>-0.1265406757400813</v>
+        <v>-0.1265406757400818</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>kgf_temerrut</t>
+          <t>bes_vazgecme</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>0.06327033787004041</v>
+        <v>-0.07361091709504318</v>
       </c>
       <c r="C44" t="n">
-        <v>-0.1265406757400813</v>
+        <v>0.07361091709504509</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>bes_vazgecme</t>
+          <t>phi</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>-0.07361091709504318</v>
+        <v>0.03464387011085701</v>
       </c>
       <c r="C45" t="n">
-        <v>0.07361091709504509</v>
+        <v>-0.06928774022171402</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>phi</t>
+          <t>onlem</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>0.03464387011085701</v>
+        <v>-0.02078632206651497</v>
       </c>
       <c r="C46" t="n">
-        <v>-0.06928774022171354</v>
+        <v>0.02078632206651306</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>onlem</t>
+          <t>prim_odeme</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>-0.02078632206651402</v>
+        <v>0</v>
       </c>
       <c r="C47" t="n">
-        <v>0.02078632206651449</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Denetim raporu, excel, bolme kazanci, banner ve model dosyalari guncellendi
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012gVZQXddJGKmSE7re5wowB
</commit_message>
<xml_diff>
--- a/kanun/EKLER_PDF/05b_Mali_Model_Excel.xlsx
+++ b/kanun/EKLER_PDF/05b_Mali_Model_Excel.xlsx
@@ -612,13 +612,13 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>350000</v>
+        <v>331000</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>700000</v>
+        <v>1096000</v>
       </c>
       <c r="F9" s="4">
         <f>INDEX(C9:E9,$D$2)</f>
@@ -626,7 +626,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Varsayım; veri talebi: GİB, SGK</t>
+          <t>Kötümser: F 3-I 268; İyimser: F 3-I 269 oranları × ILO 2025 + F 3-I 273 gayrıresmî tanımı (n_veri.py); Orta: geometrik ortalama (Claude)</t>
         </is>
       </c>
     </row>
@@ -656,14 +656,14 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Varsayım; prim sürdüğü için sonucu az etkiler</t>
+          <t>Varsayım; prim isteğe bağlı olduğundan sonucu çok etkiler</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Halen kayıtlı olanın 4/b primine devamı (1 = prim sürer)</t>
+          <t>Halen kayıtlı olanın isteğe bağlı primi sürdürme payı (0 = hiç sürdürmez)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -672,13 +672,13 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F11" s="4">
         <f>INDEX(C11:E11,$D$2)</f>
@@ -686,7 +686,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Teklif Madde 1 (p)</t>
+          <t>Teklif Madde 1 (p), 5 (o): prim isteğe bağlı; en kötü hâl 0</t>
         </is>
       </c>
     </row>
@@ -702,13 +702,13 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="F12" s="4">
         <f>INDEX(C12:E12,$D$2)</f>
@@ -716,29 +716,29 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Varsayım</t>
+          <t>Teklif Madde 1 (t): ücretli çalışan rejim dışında (F 3-I 302)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Götürü gider oranı</t>
+          <t>Tevkifat oranı (gayrisafi hasılatın)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>gider</t>
+          <t>duz_oran</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.3</v>
+        <v>0.135</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.3</v>
+        <v>0.135</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>0.3</v>
+        <v>0.135</v>
       </c>
       <c r="F13" s="4">
         <f>INDEX(C13:E13,$D$2)</f>
@@ -746,7 +746,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Teklif Madde 1 (a)</t>
+          <t>Teklif Madde 1 (e): %13,5 ile %27 arası; F 3-I 299</t>
         </is>
       </c>
     </row>
@@ -1770,7 +1770,7 @@
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
-          <t>Safi matrah</t>
+          <t>Tevkifat matrahı (gayrisafi)</t>
         </is>
       </c>
       <c r="G1" s="3" t="inlineStr">
@@ -1835,11 +1835,11 @@
         <v/>
       </c>
       <c r="F2">
-        <f>(1-Girdiler!$F$13)*D2</f>
+        <f>D2</f>
         <v/>
       </c>
       <c r="G2">
-        <f>SUMPRODUCT((F2&gt;Girdiler!$D$47:$D$51)*(F2-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F2</f>
         <v/>
       </c>
       <c r="H2">
@@ -1892,11 +1892,11 @@
         <v/>
       </c>
       <c r="F3">
-        <f>(1-Girdiler!$F$13)*D3</f>
+        <f>D3</f>
         <v/>
       </c>
       <c r="G3">
-        <f>SUMPRODUCT((F3&gt;Girdiler!$D$47:$D$51)*(F3-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F3</f>
         <v/>
       </c>
       <c r="H3">
@@ -1949,11 +1949,11 @@
         <v/>
       </c>
       <c r="F4">
-        <f>(1-Girdiler!$F$13)*D4</f>
+        <f>D4</f>
         <v/>
       </c>
       <c r="G4">
-        <f>SUMPRODUCT((F4&gt;Girdiler!$D$47:$D$51)*(F4-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F4</f>
         <v/>
       </c>
       <c r="H4">
@@ -2006,11 +2006,11 @@
         <v/>
       </c>
       <c r="F5">
-        <f>(1-Girdiler!$F$13)*D5</f>
+        <f>D5</f>
         <v/>
       </c>
       <c r="G5">
-        <f>SUMPRODUCT((F5&gt;Girdiler!$D$47:$D$51)*(F5-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F5</f>
         <v/>
       </c>
       <c r="H5">
@@ -2063,11 +2063,11 @@
         <v/>
       </c>
       <c r="F6">
-        <f>(1-Girdiler!$F$13)*D6</f>
+        <f>D6</f>
         <v/>
       </c>
       <c r="G6">
-        <f>SUMPRODUCT((F6&gt;Girdiler!$D$47:$D$51)*(F6-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F6</f>
         <v/>
       </c>
       <c r="H6">
@@ -2120,11 +2120,11 @@
         <v/>
       </c>
       <c r="F7">
-        <f>(1-Girdiler!$F$13)*D7</f>
+        <f>D7</f>
         <v/>
       </c>
       <c r="G7">
-        <f>SUMPRODUCT((F7&gt;Girdiler!$D$47:$D$51)*(F7-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F7</f>
         <v/>
       </c>
       <c r="H7">
@@ -2177,11 +2177,11 @@
         <v/>
       </c>
       <c r="F8">
-        <f>(1-Girdiler!$F$13)*D8</f>
+        <f>D8</f>
         <v/>
       </c>
       <c r="G8">
-        <f>SUMPRODUCT((F8&gt;Girdiler!$D$47:$D$51)*(F8-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F8</f>
         <v/>
       </c>
       <c r="H8">
@@ -2234,11 +2234,11 @@
         <v/>
       </c>
       <c r="F9">
-        <f>(1-Girdiler!$F$13)*D9</f>
+        <f>D9</f>
         <v/>
       </c>
       <c r="G9">
-        <f>SUMPRODUCT((F9&gt;Girdiler!$D$47:$D$51)*(F9-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F9</f>
         <v/>
       </c>
       <c r="H9">
@@ -2291,11 +2291,11 @@
         <v/>
       </c>
       <c r="F10">
-        <f>(1-Girdiler!$F$13)*D10</f>
+        <f>D10</f>
         <v/>
       </c>
       <c r="G10">
-        <f>SUMPRODUCT((F10&gt;Girdiler!$D$47:$D$51)*(F10-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F10</f>
         <v/>
       </c>
       <c r="H10">
@@ -2348,11 +2348,11 @@
         <v/>
       </c>
       <c r="F11">
-        <f>(1-Girdiler!$F$13)*D11</f>
+        <f>D11</f>
         <v/>
       </c>
       <c r="G11">
-        <f>SUMPRODUCT((F11&gt;Girdiler!$D$47:$D$51)*(F11-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F11</f>
         <v/>
       </c>
       <c r="H11">
@@ -2405,11 +2405,11 @@
         <v/>
       </c>
       <c r="F12">
-        <f>(1-Girdiler!$F$13)*D12</f>
+        <f>D12</f>
         <v/>
       </c>
       <c r="G12">
-        <f>SUMPRODUCT((F12&gt;Girdiler!$D$47:$D$51)*(F12-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F12</f>
         <v/>
       </c>
       <c r="H12">
@@ -2462,11 +2462,11 @@
         <v/>
       </c>
       <c r="F13">
-        <f>(1-Girdiler!$F$13)*D13</f>
+        <f>D13</f>
         <v/>
       </c>
       <c r="G13">
-        <f>SUMPRODUCT((F13&gt;Girdiler!$D$47:$D$51)*(F13-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F13</f>
         <v/>
       </c>
       <c r="H13">
@@ -2519,11 +2519,11 @@
         <v/>
       </c>
       <c r="F14">
-        <f>(1-Girdiler!$F$13)*D14</f>
+        <f>D14</f>
         <v/>
       </c>
       <c r="G14">
-        <f>SUMPRODUCT((F14&gt;Girdiler!$D$47:$D$51)*(F14-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F14</f>
         <v/>
       </c>
       <c r="H14">
@@ -2576,11 +2576,11 @@
         <v/>
       </c>
       <c r="F15">
-        <f>(1-Girdiler!$F$13)*D15</f>
+        <f>D15</f>
         <v/>
       </c>
       <c r="G15">
-        <f>SUMPRODUCT((F15&gt;Girdiler!$D$47:$D$51)*(F15-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F15</f>
         <v/>
       </c>
       <c r="H15">
@@ -2633,11 +2633,11 @@
         <v/>
       </c>
       <c r="F16">
-        <f>(1-Girdiler!$F$13)*D16</f>
+        <f>D16</f>
         <v/>
       </c>
       <c r="G16">
-        <f>SUMPRODUCT((F16&gt;Girdiler!$D$47:$D$51)*(F16-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F16</f>
         <v/>
       </c>
       <c r="H16">
@@ -2690,11 +2690,11 @@
         <v/>
       </c>
       <c r="F17">
-        <f>(1-Girdiler!$F$13)*D17</f>
+        <f>D17</f>
         <v/>
       </c>
       <c r="G17">
-        <f>SUMPRODUCT((F17&gt;Girdiler!$D$47:$D$51)*(F17-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F17</f>
         <v/>
       </c>
       <c r="H17">
@@ -2747,11 +2747,11 @@
         <v/>
       </c>
       <c r="F18">
-        <f>(1-Girdiler!$F$13)*D18</f>
+        <f>D18</f>
         <v/>
       </c>
       <c r="G18">
-        <f>SUMPRODUCT((F18&gt;Girdiler!$D$47:$D$51)*(F18-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F18</f>
         <v/>
       </c>
       <c r="H18">
@@ -2804,11 +2804,11 @@
         <v/>
       </c>
       <c r="F19">
-        <f>(1-Girdiler!$F$13)*D19</f>
+        <f>D19</f>
         <v/>
       </c>
       <c r="G19">
-        <f>SUMPRODUCT((F19&gt;Girdiler!$D$47:$D$51)*(F19-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F19</f>
         <v/>
       </c>
       <c r="H19">
@@ -2861,11 +2861,11 @@
         <v/>
       </c>
       <c r="F20">
-        <f>(1-Girdiler!$F$13)*D20</f>
+        <f>D20</f>
         <v/>
       </c>
       <c r="G20">
-        <f>SUMPRODUCT((F20&gt;Girdiler!$D$47:$D$51)*(F20-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F20</f>
         <v/>
       </c>
       <c r="H20">
@@ -2918,11 +2918,11 @@
         <v/>
       </c>
       <c r="F21">
-        <f>(1-Girdiler!$F$13)*D21</f>
+        <f>D21</f>
         <v/>
       </c>
       <c r="G21">
-        <f>SUMPRODUCT((F21&gt;Girdiler!$D$47:$D$51)*(F21-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F21</f>
         <v/>
       </c>
       <c r="H21">
@@ -2975,11 +2975,11 @@
         <v/>
       </c>
       <c r="F22">
-        <f>(1-Girdiler!$F$13)*D22</f>
+        <f>D22</f>
         <v/>
       </c>
       <c r="G22">
-        <f>SUMPRODUCT((F22&gt;Girdiler!$D$47:$D$51)*(F22-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F22</f>
         <v/>
       </c>
       <c r="H22">
@@ -3032,11 +3032,11 @@
         <v/>
       </c>
       <c r="F23">
-        <f>(1-Girdiler!$F$13)*D23</f>
+        <f>D23</f>
         <v/>
       </c>
       <c r="G23">
-        <f>SUMPRODUCT((F23&gt;Girdiler!$D$47:$D$51)*(F23-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F23</f>
         <v/>
       </c>
       <c r="H23">
@@ -3089,11 +3089,11 @@
         <v/>
       </c>
       <c r="F24">
-        <f>(1-Girdiler!$F$13)*D24</f>
+        <f>D24</f>
         <v/>
       </c>
       <c r="G24">
-        <f>SUMPRODUCT((F24&gt;Girdiler!$D$47:$D$51)*(F24-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F24</f>
         <v/>
       </c>
       <c r="H24">
@@ -3146,11 +3146,11 @@
         <v/>
       </c>
       <c r="F25">
-        <f>(1-Girdiler!$F$13)*D25</f>
+        <f>D25</f>
         <v/>
       </c>
       <c r="G25">
-        <f>SUMPRODUCT((F25&gt;Girdiler!$D$47:$D$51)*(F25-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F25</f>
         <v/>
       </c>
       <c r="H25">
@@ -3203,11 +3203,11 @@
         <v/>
       </c>
       <c r="F26">
-        <f>(1-Girdiler!$F$13)*D26</f>
+        <f>D26</f>
         <v/>
       </c>
       <c r="G26">
-        <f>SUMPRODUCT((F26&gt;Girdiler!$D$47:$D$51)*(F26-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F26</f>
         <v/>
       </c>
       <c r="H26">
@@ -3260,11 +3260,11 @@
         <v/>
       </c>
       <c r="F27">
-        <f>(1-Girdiler!$F$13)*D27</f>
+        <f>D27</f>
         <v/>
       </c>
       <c r="G27">
-        <f>SUMPRODUCT((F27&gt;Girdiler!$D$47:$D$51)*(F27-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F27</f>
         <v/>
       </c>
       <c r="H27">
@@ -3317,11 +3317,11 @@
         <v/>
       </c>
       <c r="F28">
-        <f>(1-Girdiler!$F$13)*D28</f>
+        <f>D28</f>
         <v/>
       </c>
       <c r="G28">
-        <f>SUMPRODUCT((F28&gt;Girdiler!$D$47:$D$51)*(F28-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F28</f>
         <v/>
       </c>
       <c r="H28">
@@ -3374,11 +3374,11 @@
         <v/>
       </c>
       <c r="F29">
-        <f>(1-Girdiler!$F$13)*D29</f>
+        <f>D29</f>
         <v/>
       </c>
       <c r="G29">
-        <f>SUMPRODUCT((F29&gt;Girdiler!$D$47:$D$51)*(F29-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F29</f>
         <v/>
       </c>
       <c r="H29">
@@ -3431,11 +3431,11 @@
         <v/>
       </c>
       <c r="F30">
-        <f>(1-Girdiler!$F$13)*D30</f>
+        <f>D30</f>
         <v/>
       </c>
       <c r="G30">
-        <f>SUMPRODUCT((F30&gt;Girdiler!$D$47:$D$51)*(F30-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F30</f>
         <v/>
       </c>
       <c r="H30">
@@ -3488,11 +3488,11 @@
         <v/>
       </c>
       <c r="F31">
-        <f>(1-Girdiler!$F$13)*D31</f>
+        <f>D31</f>
         <v/>
       </c>
       <c r="G31">
-        <f>SUMPRODUCT((F31&gt;Girdiler!$D$47:$D$51)*(F31-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F31</f>
         <v/>
       </c>
       <c r="H31">
@@ -3545,11 +3545,11 @@
         <v/>
       </c>
       <c r="F32">
-        <f>(1-Girdiler!$F$13)*D32</f>
+        <f>D32</f>
         <v/>
       </c>
       <c r="G32">
-        <f>SUMPRODUCT((F32&gt;Girdiler!$D$47:$D$51)*(F32-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F32</f>
         <v/>
       </c>
       <c r="H32">
@@ -3602,11 +3602,11 @@
         <v/>
       </c>
       <c r="F33">
-        <f>(1-Girdiler!$F$13)*D33</f>
+        <f>D33</f>
         <v/>
       </c>
       <c r="G33">
-        <f>SUMPRODUCT((F33&gt;Girdiler!$D$47:$D$51)*(F33-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F33</f>
         <v/>
       </c>
       <c r="H33">
@@ -3659,11 +3659,11 @@
         <v/>
       </c>
       <c r="F34">
-        <f>(1-Girdiler!$F$13)*D34</f>
+        <f>D34</f>
         <v/>
       </c>
       <c r="G34">
-        <f>SUMPRODUCT((F34&gt;Girdiler!$D$47:$D$51)*(F34-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F34</f>
         <v/>
       </c>
       <c r="H34">
@@ -3716,11 +3716,11 @@
         <v/>
       </c>
       <c r="F35">
-        <f>(1-Girdiler!$F$13)*D35</f>
+        <f>D35</f>
         <v/>
       </c>
       <c r="G35">
-        <f>SUMPRODUCT((F35&gt;Girdiler!$D$47:$D$51)*(F35-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F35</f>
         <v/>
       </c>
       <c r="H35">
@@ -3773,11 +3773,11 @@
         <v/>
       </c>
       <c r="F36">
-        <f>(1-Girdiler!$F$13)*D36</f>
+        <f>D36</f>
         <v/>
       </c>
       <c r="G36">
-        <f>SUMPRODUCT((F36&gt;Girdiler!$D$47:$D$51)*(F36-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F36</f>
         <v/>
       </c>
       <c r="H36">
@@ -3830,11 +3830,11 @@
         <v/>
       </c>
       <c r="F37">
-        <f>(1-Girdiler!$F$13)*D37</f>
+        <f>D37</f>
         <v/>
       </c>
       <c r="G37">
-        <f>SUMPRODUCT((F37&gt;Girdiler!$D$47:$D$51)*(F37-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F37</f>
         <v/>
       </c>
       <c r="H37">
@@ -3887,11 +3887,11 @@
         <v/>
       </c>
       <c r="F38">
-        <f>(1-Girdiler!$F$13)*D38</f>
+        <f>D38</f>
         <v/>
       </c>
       <c r="G38">
-        <f>SUMPRODUCT((F38&gt;Girdiler!$D$47:$D$51)*(F38-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F38</f>
         <v/>
       </c>
       <c r="H38">
@@ -3944,11 +3944,11 @@
         <v/>
       </c>
       <c r="F39">
-        <f>(1-Girdiler!$F$13)*D39</f>
+        <f>D39</f>
         <v/>
       </c>
       <c r="G39">
-        <f>SUMPRODUCT((F39&gt;Girdiler!$D$47:$D$51)*(F39-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F39</f>
         <v/>
       </c>
       <c r="H39">
@@ -4001,11 +4001,11 @@
         <v/>
       </c>
       <c r="F40">
-        <f>(1-Girdiler!$F$13)*D40</f>
+        <f>D40</f>
         <v/>
       </c>
       <c r="G40">
-        <f>SUMPRODUCT((F40&gt;Girdiler!$D$47:$D$51)*(F40-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F40</f>
         <v/>
       </c>
       <c r="H40">
@@ -4058,11 +4058,11 @@
         <v/>
       </c>
       <c r="F41">
-        <f>(1-Girdiler!$F$13)*D41</f>
+        <f>D41</f>
         <v/>
       </c>
       <c r="G41">
-        <f>SUMPRODUCT((F41&gt;Girdiler!$D$47:$D$51)*(F41-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F41</f>
         <v/>
       </c>
       <c r="H41">
@@ -4115,11 +4115,11 @@
         <v/>
       </c>
       <c r="F42">
-        <f>(1-Girdiler!$F$13)*D42</f>
+        <f>D42</f>
         <v/>
       </c>
       <c r="G42">
-        <f>SUMPRODUCT((F42&gt;Girdiler!$D$47:$D$51)*(F42-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F42</f>
         <v/>
       </c>
       <c r="H42">
@@ -4172,11 +4172,11 @@
         <v/>
       </c>
       <c r="F43">
-        <f>(1-Girdiler!$F$13)*D43</f>
+        <f>D43</f>
         <v/>
       </c>
       <c r="G43">
-        <f>SUMPRODUCT((F43&gt;Girdiler!$D$47:$D$51)*(F43-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F43</f>
         <v/>
       </c>
       <c r="H43">
@@ -4229,11 +4229,11 @@
         <v/>
       </c>
       <c r="F44">
-        <f>(1-Girdiler!$F$13)*D44</f>
+        <f>D44</f>
         <v/>
       </c>
       <c r="G44">
-        <f>SUMPRODUCT((F44&gt;Girdiler!$D$47:$D$51)*(F44-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F44</f>
         <v/>
       </c>
       <c r="H44">
@@ -4286,11 +4286,11 @@
         <v/>
       </c>
       <c r="F45">
-        <f>(1-Girdiler!$F$13)*D45</f>
+        <f>D45</f>
         <v/>
       </c>
       <c r="G45">
-        <f>SUMPRODUCT((F45&gt;Girdiler!$D$47:$D$51)*(F45-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F45</f>
         <v/>
       </c>
       <c r="H45">
@@ -4343,11 +4343,11 @@
         <v/>
       </c>
       <c r="F46">
-        <f>(1-Girdiler!$F$13)*D46</f>
+        <f>D46</f>
         <v/>
       </c>
       <c r="G46">
-        <f>SUMPRODUCT((F46&gt;Girdiler!$D$47:$D$51)*(F46-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F46</f>
         <v/>
       </c>
       <c r="H46">
@@ -4400,11 +4400,11 @@
         <v/>
       </c>
       <c r="F47">
-        <f>(1-Girdiler!$F$13)*D47</f>
+        <f>D47</f>
         <v/>
       </c>
       <c r="G47">
-        <f>SUMPRODUCT((F47&gt;Girdiler!$D$47:$D$51)*(F47-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F47</f>
         <v/>
       </c>
       <c r="H47">
@@ -4457,11 +4457,11 @@
         <v/>
       </c>
       <c r="F48">
-        <f>(1-Girdiler!$F$13)*D48</f>
+        <f>D48</f>
         <v/>
       </c>
       <c r="G48">
-        <f>SUMPRODUCT((F48&gt;Girdiler!$D$47:$D$51)*(F48-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F48</f>
         <v/>
       </c>
       <c r="H48">
@@ -4514,11 +4514,11 @@
         <v/>
       </c>
       <c r="F49">
-        <f>(1-Girdiler!$F$13)*D49</f>
+        <f>D49</f>
         <v/>
       </c>
       <c r="G49">
-        <f>SUMPRODUCT((F49&gt;Girdiler!$D$47:$D$51)*(F49-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F49</f>
         <v/>
       </c>
       <c r="H49">
@@ -4571,11 +4571,11 @@
         <v/>
       </c>
       <c r="F50">
-        <f>(1-Girdiler!$F$13)*D50</f>
+        <f>D50</f>
         <v/>
       </c>
       <c r="G50">
-        <f>SUMPRODUCT((F50&gt;Girdiler!$D$47:$D$51)*(F50-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F50</f>
         <v/>
       </c>
       <c r="H50">
@@ -4628,11 +4628,11 @@
         <v/>
       </c>
       <c r="F51">
-        <f>(1-Girdiler!$F$13)*D51</f>
+        <f>D51</f>
         <v/>
       </c>
       <c r="G51">
-        <f>SUMPRODUCT((F51&gt;Girdiler!$D$47:$D$51)*(F51-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F51</f>
         <v/>
       </c>
       <c r="H51">
@@ -4685,11 +4685,11 @@
         <v/>
       </c>
       <c r="F52">
-        <f>(1-Girdiler!$F$13)*D52</f>
+        <f>D52</f>
         <v/>
       </c>
       <c r="G52">
-        <f>SUMPRODUCT((F52&gt;Girdiler!$D$47:$D$51)*(F52-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F52</f>
         <v/>
       </c>
       <c r="H52">
@@ -4742,11 +4742,11 @@
         <v/>
       </c>
       <c r="F53">
-        <f>(1-Girdiler!$F$13)*D53</f>
+        <f>D53</f>
         <v/>
       </c>
       <c r="G53">
-        <f>SUMPRODUCT((F53&gt;Girdiler!$D$47:$D$51)*(F53-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F53</f>
         <v/>
       </c>
       <c r="H53">
@@ -4799,11 +4799,11 @@
         <v/>
       </c>
       <c r="F54">
-        <f>(1-Girdiler!$F$13)*D54</f>
+        <f>D54</f>
         <v/>
       </c>
       <c r="G54">
-        <f>SUMPRODUCT((F54&gt;Girdiler!$D$47:$D$51)*(F54-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F54</f>
         <v/>
       </c>
       <c r="H54">
@@ -4856,11 +4856,11 @@
         <v/>
       </c>
       <c r="F55">
-        <f>(1-Girdiler!$F$13)*D55</f>
+        <f>D55</f>
         <v/>
       </c>
       <c r="G55">
-        <f>SUMPRODUCT((F55&gt;Girdiler!$D$47:$D$51)*(F55-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F55</f>
         <v/>
       </c>
       <c r="H55">
@@ -4913,11 +4913,11 @@
         <v/>
       </c>
       <c r="F56">
-        <f>(1-Girdiler!$F$13)*D56</f>
+        <f>D56</f>
         <v/>
       </c>
       <c r="G56">
-        <f>SUMPRODUCT((F56&gt;Girdiler!$D$47:$D$51)*(F56-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F56</f>
         <v/>
       </c>
       <c r="H56">
@@ -4970,11 +4970,11 @@
         <v/>
       </c>
       <c r="F57">
-        <f>(1-Girdiler!$F$13)*D57</f>
+        <f>D57</f>
         <v/>
       </c>
       <c r="G57">
-        <f>SUMPRODUCT((F57&gt;Girdiler!$D$47:$D$51)*(F57-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F57</f>
         <v/>
       </c>
       <c r="H57">
@@ -5027,11 +5027,11 @@
         <v/>
       </c>
       <c r="F58">
-        <f>(1-Girdiler!$F$13)*D58</f>
+        <f>D58</f>
         <v/>
       </c>
       <c r="G58">
-        <f>SUMPRODUCT((F58&gt;Girdiler!$D$47:$D$51)*(F58-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F58</f>
         <v/>
       </c>
       <c r="H58">
@@ -5084,11 +5084,11 @@
         <v/>
       </c>
       <c r="F59">
-        <f>(1-Girdiler!$F$13)*D59</f>
+        <f>D59</f>
         <v/>
       </c>
       <c r="G59">
-        <f>SUMPRODUCT((F59&gt;Girdiler!$D$47:$D$51)*(F59-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F59</f>
         <v/>
       </c>
       <c r="H59">
@@ -5141,11 +5141,11 @@
         <v/>
       </c>
       <c r="F60">
-        <f>(1-Girdiler!$F$13)*D60</f>
+        <f>D60</f>
         <v/>
       </c>
       <c r="G60">
-        <f>SUMPRODUCT((F60&gt;Girdiler!$D$47:$D$51)*(F60-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F60</f>
         <v/>
       </c>
       <c r="H60">
@@ -5198,11 +5198,11 @@
         <v/>
       </c>
       <c r="F61">
-        <f>(1-Girdiler!$F$13)*D61</f>
+        <f>D61</f>
         <v/>
       </c>
       <c r="G61">
-        <f>SUMPRODUCT((F61&gt;Girdiler!$D$47:$D$51)*(F61-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>Girdiler!$F$13*F61</f>
         <v/>
       </c>
       <c r="H61">
@@ -5449,7 +5449,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Not: prim sürekliliği (prim_devam=1) ile kırılma noktası yoktur; s=1 için Python varyantı Senaryolar_Python sayfasındadır.</t>
+          <t>Not: prim_devam=0 en kötü hâldir (eski kayıtlıların primi hiç sürmez); varyantlar Senaryolar_Python sayfasındadır.</t>
         </is>
       </c>
     </row>
@@ -5464,7 +5464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:C49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -5501,10 +5501,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1.084463422748595</v>
+        <v>-2.013885121244206</v>
       </c>
       <c r="C4" t="n">
-        <v>2.986259536424468</v>
+        <v>-6.41445985704332</v>
       </c>
     </row>
     <row r="5">
@@ -5514,10 +5514,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.863742829232634</v>
+        <v>1.318681980023</v>
       </c>
       <c r="C5" t="n">
-        <v>14.45167175395206</v>
+        <v>3.69521576662539</v>
       </c>
     </row>
     <row r="6">
@@ -5527,10 +5527,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>14.18537328138288</v>
+        <v>23.71682554050645</v>
       </c>
       <c r="C6" t="n">
-        <v>42.73259043346012</v>
+        <v>71.64972496970631</v>
       </c>
     </row>
     <row r="8">
@@ -5543,405 +5543,420 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>G0 Seçilen: kapısız, halen kayıtlı olanın 4/b primi sürer (s=0,15)</t>
+          <t>V0 Baz: %13,5; eski kayıtlıların primi hiç sürmez</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>4.863742829232634</v>
+        <v>1.318681980023</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>G1 Prim sürekliliği olmasaydı (kapısız, s=0,15)</t>
+          <t>V1 Eski kayıtlıların %50'si primi sürdürür</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-1.087615170767367</v>
+        <v>4.132824120023001</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>G2 Önceki karar: 24 ay giriş kapısı (s=0,05, prim sürekliliği yok)</t>
+          <t>V2 %75'i sürdürür</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>3.440481618561076</v>
+        <v>5.539895190023</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>G3 Harici öneri: düz %15 (%5 prim payı), hibe yok, kapısız (s=0,15)</t>
+          <t>V3 Hepsi sürdürür</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1.823954910190622</v>
+        <v>6.946966260023002</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>G4 Seçilen, herkes geçse (s=1,00)</t>
+          <t>V4 Oran %20</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1.075453047078635</v>
+        <v>5.605830913815579</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>G5 Seçilen + 90 gün prim hibesi yok</t>
+          <t>V6 Oran %27 (üst sınır)</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>5.2231600036498</v>
+        <v>10.23467206349843</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>G6 Seçilen + donanım KDV mahsubu yok</t>
+          <t>V7 Ücretli çalışana izin verilseydi (u=%20)</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>5.490252664609205</v>
+        <v>0.3955031889298513</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>G7 Seçilen + (e) bendi yok: düz %10,5</t>
+          <t>V8 SGK tahsil oranı %50</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>4.29473043759288</v>
+        <v>3.429288585022999</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>G8 Seçilen + götürü gider %25</t>
+          <t>V9 SGK tahsil oranı %100</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>5.519902244678498</v>
+        <v>-0.08838908997700055</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>V10 Halen kayıtlıların hepsi geçse (s=%100)</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>-35.08074749647865</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>V11 90 gün prim hibesi olmasaydı</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1.658587936400376</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>V12 Donanım KDV mahsubu olmasaydı</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1.936435777712903</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Kırılma noktası s* (Orta)</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>yok</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+      <c r="B22" t="n">
+        <v>0.1807938805398902</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Monte Carlo (4000 deneme), 4. yıl net (mlr TL)</t>
         </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>P5</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>1.371685259209676</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>P10</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>1.816043653111378</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>P25</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>2.740448089415021</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>P50</t>
+          <t>P5</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>4.210833232420195</v>
+        <v>-6.355437545210761</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>P75</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>6.348701487779011</v>
+        <v>-3.380972462056701</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>P90</t>
+          <t>P25</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>9.050144277377949</v>
+        <v>0.3984784252397677</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>P95</t>
+          <t>P50</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>11.31276202009183</v>
+        <v>2.93701569013757</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>P(net&gt;0)</t>
+          <t>P75</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>0.99875</v>
+        <v>5.812795204092121</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>P90</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>9.342409413022768</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>Tornado (Orta tabanı, 4. yıl net değişimi, mlr TL)</t>
-        </is>
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>P95</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>12.12628166050324</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>n_toplam</t>
+          <t>P(net&gt;0)</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>-2.807853045275791</v>
-      </c>
-      <c r="C32" t="n">
-        <v>4.913742829232634</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>medyan_W</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>-1.816846647234291</v>
-      </c>
-      <c r="C33" t="n">
-        <v>2.027565172759112</v>
+        <v>0.77025</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>s_kayitli</t>
-        </is>
-      </c>
-      <c r="B34" t="n">
-        <v>0.8407871839926644</v>
-      </c>
-      <c r="C34" t="n">
-        <v>-0.2802623946642227</v>
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Tornado (Orta tabanı, 4. yıl net değişimi, mlr TL)</t>
+        </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>uyum_ucretli</t>
+          <t>duz_oran</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>0.5857025562826614</v>
+        <v>-1.964913826520587</v>
       </c>
       <c r="C35" t="n">
-        <v>-0.5857025562826629</v>
+        <v>8.915990083475434</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>marj</t>
+          <t>s_kayitli</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>0.5589775689572811</v>
+        <v>6.42342873114735</v>
       </c>
       <c r="C36" t="n">
-        <v>-0.5786323428758425</v>
+        <v>-2.141142910382449</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>u_ucretli</t>
+          <t>prim_devam</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>0.4880854635688839</v>
+        <v>0</v>
       </c>
       <c r="C37" t="n">
-        <v>-0.4880854635688858</v>
+        <v>5.628284280000002</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>sigma</t>
+          <t>n_toplam</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>-0.4620656689140339</v>
+        <v>-0.9551828924027577</v>
       </c>
       <c r="C38" t="n">
-        <v>0.02112601201078796</v>
+        <v>3.163268020294853</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>kdv_donanim_pay</t>
+          <t>prim_odeme</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>0.3132549176882858</v>
+        <v>2.814142140000001</v>
       </c>
       <c r="C39" t="n">
-        <v>-0.3132549176882877</v>
+        <v>-1.40707107</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>r_marj_ucretli</t>
+          <t>medyan_W</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>0.2530813514801616</v>
+        <v>-2.372042154910663</v>
       </c>
       <c r="C40" t="n">
-        <v>-0.2892358302630443</v>
+        <v>2.463885342496412</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>myo_uygun</t>
+          <t>sigma</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>0.2567265531551189</v>
+        <v>-0.3384366074561423</v>
       </c>
       <c r="C41" t="n">
-        <v>-0.2567265531551171</v>
+        <v>-0.1350771362789137</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>kgf_alim</t>
+          <t>kdv_donanim_pay</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>0.07592440544404792</v>
+        <v>0.3088768988449516</v>
       </c>
       <c r="C42" t="n">
-        <v>-0.1265406757400818</v>
+        <v>-0.3088768988449515</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>kgf_temerrut</t>
+          <t>marj</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>0.06327033787003994</v>
+        <v>0.2516794350287991</v>
       </c>
       <c r="C43" t="n">
-        <v>-0.1265406757400818</v>
+        <v>-0.2702672355060652</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>bes_vazgecme</t>
+          <t>myo_uygun</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>-0.07361091709504318</v>
+        <v>0.2427899688409824</v>
       </c>
       <c r="C44" t="n">
-        <v>0.07361091709504509</v>
+        <v>-0.2427899688409824</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>phi</t>
+          <t>kgf_alim</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>0.03464387011085701</v>
+        <v>0.07180279486280036</v>
       </c>
       <c r="C45" t="n">
-        <v>-0.06928774022171402</v>
+        <v>-0.1196713247713342</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>onlem</t>
+          <t>kgf_temerrut</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>-0.02078632206651497</v>
+        <v>0.05983566238566685</v>
       </c>
       <c r="C46" t="n">
-        <v>0.02078632206651306</v>
+        <v>-0.1196713247713342</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>prim_odeme</t>
+          <t>bes_vazgecme</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>0</v>
+        <v>-0.08308609119838332</v>
       </c>
       <c r="C47" t="n">
-        <v>0</v>
+        <v>0.08308609119838332</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>phi</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>0.02752440469740677</v>
+      </c>
+      <c r="C48" t="n">
+        <v>-0.05504880939481378</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>onlem</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>-0.01651464281844425</v>
+      </c>
+      <c r="C49" t="n">
+        <v>0.01651464281844401</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
F 3-I 304: gelire bagli prim (gecim haddi, tam prim 6 asgari), maasli kisiti geri alindi, model/genc/excel/resim paketi yenilendi, tavan ustu bolme secenekleri
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012gVZQXddJGKmSE7re5wowB
</commit_message>
<xml_diff>
--- a/kanun/EKLER_PDF/05b_Mali_Model_Excel.xlsx
+++ b/kanun/EKLER_PDF/05b_Mali_Model_Excel.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -663,22 +663,22 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Halen kayıtlı olanın isteğe bağlı primi sürdürme payı (0 = hiç sürdürmez)</t>
+          <t>Gelire bağlı prim: tam prim eşiği (brüt asgari ücret katı)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>prim_devam</t>
+          <t>prim_k</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F11" s="4">
         <f>INDEX(C11:E11,$D$2)</f>
@@ -686,29 +686,29 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Teklif Madde 1 (p), 5 (o): prim isteğe bağlı; en kötü hâl 0</t>
+          <t>Teklif Madde 5 (o); genç simülasyonunda seçildi (prim_esigi_out2.txt); F 3-I 304</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Ücretli ek gelir payı (u)</t>
+          <t>Tam prim tutarı (TL/ay)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>u_ucretli</t>
+          <t>prim_ay</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0</v>
+        <v>11808.25</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0</v>
+        <v>11808.25</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>0</v>
+        <v>11808.25</v>
       </c>
       <c r="F12" s="4">
         <f>INDEX(C12:E12,$D$2)</f>
@@ -716,29 +716,29 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Teklif Madde 1 (t): ücretli çalışan rejim dışında (F 3-I 302)</t>
+          <t>5510 m.81: 33.030 x %35,75</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Tevkifat oranı (gayrisafi hasılatın)</t>
+          <t>Gelire bağlı primin tahsil oranı</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>duz_oran</t>
+          <t>prim_toplama</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.135</v>
+        <v>1</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.135</v>
+        <v>1</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>0.135</v>
+        <v>1</v>
       </c>
       <c r="F13" s="4">
         <f>INDEX(C13:E13,$D$2)</f>
@@ -746,29 +746,29 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Teklif Madde 1 (e): %13,5 ile %27 arası; F 3-I 299</t>
+          <t>Tevkifatla birlikte kaynakta kesilir (tasarım); ölçülmemiş</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>BES aktarım oranı (tevkifatın)</t>
+          <t>Eski kayıtlıların sabit primi sürdürme payı (0 = hiç sürdürmez)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>bes</t>
+          <t>prim_devam</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="F14" s="4">
         <f>INDEX(C14:E14,$D$2)</f>
@@ -776,29 +776,29 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Teklif Madde 9</t>
+          <t>Sabit prim kalktığı için 0</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Devlet katkısı oranı</t>
+          <t>Maaşlı çalışanın mikro mükellef olma payı (u)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>devlet_katki</t>
+          <t>u_ucretli</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.2</v>
+        <v>0.25</v>
       </c>
       <c r="D15" s="2" t="n">
         <v>0.2</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>0.2</v>
+        <v>0.15</v>
       </c>
       <c r="F15" s="4">
         <f>INDEX(C15:E15,$D$2)</f>
@@ -806,29 +806,29 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>4632 Ek 1 + 10811 sayılı Karar (ikincil)</t>
+          <t>Varsayım; maaşlı isterse girer (F 3-I 304)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>BES vazgeçme payı</t>
+          <t>Tevkifat oranı (gayrisafi hasılatın)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>bes_vazgecme</t>
+          <t>duz_oran</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.2</v>
+        <v>0.135</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0.35</v>
+        <v>0.135</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>0.5</v>
+        <v>0.135</v>
       </c>
       <c r="F16" s="4">
         <f>INDEX(C16:E16,$D$2)</f>
@@ -836,29 +836,29 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Varsayım</t>
+          <t>Teklif Madde 1 (e): %13,5 ile %27 arası; F 3-I 299</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>MYÖ prim oranı</t>
+          <t>BES aktarım oranı (tevkifatın)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>myo_oran</t>
+          <t>bes</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.21</v>
+        <v>0.03</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>0.21</v>
+        <v>0.03</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>0.21</v>
+        <v>0.03</v>
       </c>
       <c r="F17" s="4">
         <f>INDEX(C17:E17,$D$2)</f>
@@ -866,29 +866,29 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>5510 m.81</t>
+          <t>Teklif Madde 9</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Hibe prim süresi (ay)</t>
+          <t>Devlet katkısı oranı</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>myo_gun_ay</t>
+          <t>devlet_katki</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>3</v>
+        <v>0.2</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>3</v>
+        <v>0.2</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>3</v>
+        <v>0.2</v>
       </c>
       <c r="F18" s="4">
         <f>INDEX(C18:E18,$D$2)</f>
@@ -896,29 +896,29 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Teklif 5510 Ek 25 (90 gün)</t>
+          <t>4632 Ek 1 + 10811 sayılı Karar (ikincil)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>90 gün primi hak edenlerin payı (çakışmasız)</t>
+          <t>BES vazgeçme payı</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>myo_uygun</t>
+          <t>bes_vazgecme</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="D19" s="2" t="n">
         <v>0.35</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="F19" s="4">
         <f>INDEX(C19:E19,$D$2)</f>
@@ -933,22 +933,22 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Donanım alan payı</t>
+          <t>MYÖ prim oranı</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>kdv_donanim_pay</t>
+          <t>myo_oran</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>0.5</v>
+        <v>0.21</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>0.4</v>
+        <v>0.21</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>0.3</v>
+        <v>0.21</v>
       </c>
       <c r="F20" s="4">
         <f>INDEX(C20:E20,$D$2)</f>
@@ -956,29 +956,29 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Varsayım</t>
+          <t>5510 m.81</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Yıllık donanım KDV ortalaması (TL)</t>
+          <t>Hibe prim süresi (ay)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>kdv_donanim_kdv</t>
+          <t>myo_gun_ay</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>5000</v>
+        <v>3</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>5000</v>
+        <v>3</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>5000</v>
+        <v>3</v>
       </c>
       <c r="F21" s="4">
         <f>INDEX(C21:E21,$D$2)</f>
@@ -986,29 +986,29 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Varsayım</t>
+          <t>Teklif 5510 Ek 25 (90 gün)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>KDV mahsup üst sınırı (tevkifatın oranı)</t>
+          <t>90 gün primi hak edenlerin payı (çakışmasız)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>kdv_mahsup_tavan</t>
+          <t>myo_uygun</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
         <v>0.5</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>0.5</v>
+        <v>0.35</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="F22" s="4">
         <f>INDEX(C22:E22,$D$2)</f>
@@ -1016,29 +1016,29 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Teklif Madde 3 önerisi</t>
+          <t>Varsayım</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Eski rejimde kâr marjı</t>
+          <t>Donanım alan payı</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>marj</t>
+          <t>kdv_donanim_pay</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
         <v>0.5</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="F23" s="4">
         <f>INDEX(C23:E23,$D$2)</f>
@@ -1053,22 +1053,22 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Eski 4/b yıllık asgari prim (TL)</t>
+          <t>Yıllık donanım KDV ortalaması (TL)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>prim_eski</t>
+          <t>kdv_donanim_kdv</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>141699</v>
+        <v>5000</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>141699</v>
+        <v>5000</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>141699</v>
+        <v>5000</v>
       </c>
       <c r="F24" s="4">
         <f>INDEX(C24:E24,$D$2)</f>
@@ -1076,29 +1076,29 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>33.030×%35,75×12</t>
+          <t>Varsayım</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Eski prim ödeme oranı</t>
+          <t>KDV mahsup üst sınırı (tevkifatın oranı)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>prim_odeme</t>
+          <t>kdv_mahsup_tavan</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="F25" s="4">
         <f>INDEX(C25:E25,$D$2)</f>
@@ -1106,29 +1106,29 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Varsayım</t>
+          <t>Teklif Madde 3 önerisi</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Ücretlinin marjinal oranı</t>
+          <t>Eski rejimde kâr marjı</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>r_marj_ucretli</t>
+          <t>marj</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>0.27</v>
+        <v>0.5</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>0.27</v>
+        <v>0.5</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>0.27</v>
+        <v>0.5</v>
       </c>
       <c r="F26" s="4">
         <f>INDEX(C26:E26,$D$2)</f>
@@ -1143,22 +1143,22 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Ücretlinin eski rejimde uyum oranı</t>
+          <t>Eski 4/b yıllık asgari prim (TL)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>uyum_ucretli</t>
+          <t>prim_eski</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>0.5</v>
+        <v>141699</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>0.5</v>
+        <v>141699</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>0.5</v>
+        <v>141699</v>
       </c>
       <c r="F27" s="4">
         <f>INDEX(C27:E27,$D$2)</f>
@@ -1166,29 +1166,29 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Varsayım</t>
+          <t>33.030×%35,75×12</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Kurumsal alıcı payı</t>
+          <t>Eski prim ödeme oranı</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>kurumsal_pay</t>
+          <t>prim_odeme</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="F28" s="4">
         <f>INDEX(C28:E28,$D$2)</f>
@@ -1203,22 +1203,22 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Kurumlar vergisi oranı</t>
+          <t>Ücretlinin marjinal oranı</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>kv</t>
+          <t>r_marj_ucretli</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>0.25</v>
+        <v>0.27</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>0.25</v>
+        <v>0.27</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>0.25</v>
+        <v>0.27</v>
       </c>
       <c r="F29" s="4">
         <f>INDEX(C29:E29,$D$2)</f>
@@ -1226,29 +1226,29 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Varsayım (kanunda %25)</t>
+          <t>Varsayım</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Sahte fatura payı (kurumsal akışta, φ)</t>
+          <t>Ücretlinin eski rejimde uyum oranı</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>phi</t>
+          <t>uyum_ucretli</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>0.02</v>
+        <v>0.5</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>0.01</v>
+        <v>0.5</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>0.005</v>
+        <v>0.5</v>
       </c>
       <c r="F30" s="4">
         <f>INDEX(C30:E30,$D$2)</f>
@@ -1263,19 +1263,19 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Önlem etkinliği</t>
+          <t>Kurumsal alıcı payı</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>onlem</t>
+          <t>kurumsal_pay</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="E31" s="2" t="n">
         <v>0.7</v>
@@ -1293,22 +1293,22 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>KGF kullanım oranı</t>
+          <t>Kurumlar vergisi oranı</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>kgf_alim</t>
+          <t>kv</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
-        <v>0.08</v>
+        <v>0.25</v>
       </c>
       <c r="D32" s="2" t="n">
-        <v>0.05</v>
+        <v>0.25</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>0.03</v>
+        <v>0.25</v>
       </c>
       <c r="F32" s="4">
         <f>INDEX(C32:E32,$D$2)</f>
@@ -1316,29 +1316,29 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Varsayım</t>
+          <t>Varsayım (kanunda %25)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>KGF temerrüt oranı</t>
+          <t>Sahte fatura payı (kurumsal akışta, φ)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>kgf_temerrut</t>
+          <t>phi</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
-        <v>0.15</v>
+        <v>0.02</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>0.1</v>
+        <v>0.01</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>0.06</v>
+        <v>0.005</v>
       </c>
       <c r="F33" s="4">
         <f>INDEX(C33:E33,$D$2)</f>
@@ -1353,22 +1353,22 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>KGF kurtarma oranı</t>
+          <t>Önlem etkinliği</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>kgf_kurtarma</t>
+          <t>onlem</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
         <v>0.3</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="F34" s="4">
         <f>INDEX(C34:E34,$D$2)</f>
@@ -1383,22 +1383,22 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Kefalet tutarı (hasılatın payı)</t>
+          <t>KGF kullanım oranı</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>kgf_pay</t>
+          <t>kgf_alim</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
-        <v>0.5</v>
+        <v>0.08</v>
       </c>
       <c r="D35" s="2" t="n">
-        <v>0.5</v>
+        <v>0.05</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>0.5</v>
+        <v>0.03</v>
       </c>
       <c r="F35" s="4">
         <f>INDEX(C35:E35,$D$2)</f>
@@ -1406,29 +1406,29 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Teklif Madde 8</t>
+          <t>Varsayım</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>PTT UETS birim gideri (TL)</t>
+          <t>KGF temerrüt oranı</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>ptt_birim</t>
+          <t>kgf_temerrut</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>50</v>
+        <v>0.15</v>
       </c>
       <c r="D36" s="2" t="n">
-        <v>50</v>
+        <v>0.1</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>50</v>
+        <v>0.06</v>
       </c>
       <c r="F36" s="4">
         <f>INDEX(C36:E36,$D$2)</f>
@@ -1443,22 +1443,22 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>UETS tahsis payı</t>
+          <t>KGF kurtarma oranı</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ptt_pay</t>
+          <t>kgf_kurtarma</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
-        <v>0.8</v>
+        <v>0.3</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>0.8</v>
+        <v>0.3</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>0.8</v>
+        <v>0.3</v>
       </c>
       <c r="F37" s="4">
         <f>INDEX(C37:E37,$D$2)</f>
@@ -1473,22 +1473,22 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Tek seferlik BT gideri (TL)</t>
+          <t>Kefalet tutarı (hasılatın payı)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>bt_tek</t>
+          <t>kgf_pay</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
-        <v>250000000</v>
+        <v>0.5</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>250000000</v>
+        <v>0.5</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>250000000</v>
+        <v>0.5</v>
       </c>
       <c r="F38" s="4">
         <f>INDEX(C38:E38,$D$2)</f>
@@ -1496,29 +1496,29 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Varsayım</t>
+          <t>Teklif Madde 8</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Yıllık BT işletme gideri (TL)</t>
+          <t>PTT UETS birim gideri (TL)</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>bt_yillik</t>
+          <t>ptt_birim</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
-        <v>50000000</v>
+        <v>50</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>50000000</v>
+        <v>50</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>50000000</v>
+        <v>50</v>
       </c>
       <c r="F39" s="4">
         <f>INDEX(C39:E39,$D$2)</f>
@@ -1533,22 +1533,22 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>İtiraz oranı</t>
+          <t>UETS tahsis payı</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>itiraz_oran</t>
+          <t>ptt_pay</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
-        <v>0.04</v>
+        <v>0.8</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>0.04</v>
+        <v>0.8</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>0.04</v>
+        <v>0.8</v>
       </c>
       <c r="F40" s="4">
         <f>INDEX(C40:E40,$D$2)</f>
@@ -1563,22 +1563,22 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>İtiraz birim gideri (TL)</t>
+          <t>Tek seferlik BT gideri (TL)</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>itiraz_maliyet</t>
+          <t>bt_tek</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
-        <v>2000</v>
+        <v>250000000</v>
       </c>
       <c r="D41" s="2" t="n">
-        <v>2000</v>
+        <v>250000000</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>2000</v>
+        <v>250000000</v>
       </c>
       <c r="F41" s="4">
         <f>INDEX(C41:E41,$D$2)</f>
@@ -1593,22 +1593,22 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Denetim gideri (brüt tevkifatın oranı)</t>
+          <t>Yıllık BT işletme gideri (TL)</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>denetim</t>
+          <t>bt_yillik</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
-        <v>0.01</v>
+        <v>50000000</v>
       </c>
       <c r="D42" s="2" t="n">
-        <v>0.01</v>
+        <v>50000000</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>0.01</v>
+        <v>50000000</v>
       </c>
       <c r="F42" s="4">
         <f>INDEX(C42:E42,$D$2)</f>
@@ -1620,104 +1620,146 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>İtiraz oranı</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>itiraz_oran</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="D43" s="2" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="E43" s="2" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="F43" s="4">
+        <f>INDEX(C43:E43,$D$2)</f>
+        <v/>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Varsayım</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>İtiraz birim gideri (TL)</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>itiraz_maliyet</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D44" s="2" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E44" s="2" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F44" s="4">
+        <f>INDEX(C44:E44,$D$2)</f>
+        <v/>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Varsayım</t>
+        </is>
+      </c>
+    </row>
     <row r="45">
-      <c r="A45" s="4" t="inlineStr">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Denetim gideri (brüt tevkifatın oranı)</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>denetim</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D45" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E45" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F45" s="4">
+        <f>INDEX(C45:E45,$D$2)</f>
+        <v/>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Varsayım</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
         <is>
           <t>GVK m.103 tarifesi (2026 parantez içi tutarlar)</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
         <is>
           <t>Dilim üst sınırı (TL)</t>
         </is>
       </c>
-      <c r="B46" s="4" t="inlineStr">
+      <c r="B49" s="4" t="inlineStr">
         <is>
           <t>Oran</t>
         </is>
       </c>
-      <c r="C46" s="4" t="inlineStr">
+      <c r="C49" s="4" t="inlineStr">
         <is>
           <t>Artış (Δ)</t>
         </is>
       </c>
-      <c r="D46" s="4" t="inlineStr">
+      <c r="D49" s="4" t="inlineStr">
         <is>
           <t>Alt sınır</t>
         </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="n">
-        <v>190000</v>
-      </c>
-      <c r="B47" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="C47">
-        <f>B47</f>
-        <v/>
-      </c>
-      <c r="D47" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="n">
-        <v>400000</v>
-      </c>
-      <c r="B48" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="C48">
-        <f>B48-B47</f>
-        <v/>
-      </c>
-      <c r="D48">
-        <f>A47</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="B49" t="n">
-        <v>0.27</v>
-      </c>
-      <c r="C49">
-        <f>B49-B48</f>
-        <v/>
-      </c>
-      <c r="D49">
-        <f>A48</f>
-        <v/>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>5300000</v>
+        <v>190000</v>
       </c>
       <c r="B50" t="n">
-        <v>0.35</v>
+        <v>0.15</v>
       </c>
       <c r="C50">
-        <f>B50-B49</f>
-        <v/>
-      </c>
-      <c r="D50">
-        <f>A49</f>
-        <v/>
+        <f>B50</f>
+        <v/>
+      </c>
+      <c r="D50" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>1000000000000</v>
+        <v>400000</v>
       </c>
       <c r="B51" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="C51">
         <f>B51-B50</f>
@@ -1725,6 +1767,54 @@
       </c>
       <c r="D51">
         <f>A50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="B52" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="C52">
+        <f>B52-B51</f>
+        <v/>
+      </c>
+      <c r="D52">
+        <f>A51</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>5300000</v>
+      </c>
+      <c r="B53" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="C53">
+        <f>B53-B52</f>
+        <v/>
+      </c>
+      <c r="D53">
+        <f>A52</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>1000000000000</v>
+      </c>
+      <c r="B54" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C54">
+        <f>B54-B53</f>
+        <v/>
+      </c>
+      <c r="D54">
+        <f>A53</f>
         <v/>
       </c>
     </row>
@@ -1739,7 +1829,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N61"/>
+  <dimension ref="A1:O61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1813,6 +1903,11 @@
           <t>Eski vergi (ücretli)</t>
         </is>
       </c>
+      <c r="O1" s="3" t="inlineStr">
+        <is>
+          <t>Gelire bağlı yeni prim</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -1839,7 +1934,7 @@
         <v/>
       </c>
       <c r="G2">
-        <f>Girdiler!$F$13*F2</f>
+        <f>Girdiler!$F$16*F2</f>
         <v/>
       </c>
       <c r="H2">
@@ -1847,27 +1942,31 @@
         <v/>
       </c>
       <c r="I2">
-        <f>Girdiler!$F$14*G2*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G2*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J2">
-        <f>IF(D2&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D2&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K2">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G2,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G2,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L2">
-        <f>SUMPRODUCT((Girdiler!$F$23*D2&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D2-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D2&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D2-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M2">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N2">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D2</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D2</f>
+        <v/>
+      </c>
+      <c r="O2">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D2-G2)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -1896,7 +1995,7 @@
         <v/>
       </c>
       <c r="G3">
-        <f>Girdiler!$F$13*F3</f>
+        <f>Girdiler!$F$16*F3</f>
         <v/>
       </c>
       <c r="H3">
@@ -1904,27 +2003,31 @@
         <v/>
       </c>
       <c r="I3">
-        <f>Girdiler!$F$14*G3*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G3*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J3">
-        <f>IF(D3&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D3&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K3">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G3,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G3,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L3">
-        <f>SUMPRODUCT((Girdiler!$F$23*D3&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D3-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D3&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D3-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M3">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N3">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D3</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D3</f>
+        <v/>
+      </c>
+      <c r="O3">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D3-G3)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -1953,7 +2056,7 @@
         <v/>
       </c>
       <c r="G4">
-        <f>Girdiler!$F$13*F4</f>
+        <f>Girdiler!$F$16*F4</f>
         <v/>
       </c>
       <c r="H4">
@@ -1961,27 +2064,31 @@
         <v/>
       </c>
       <c r="I4">
-        <f>Girdiler!$F$14*G4*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G4*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J4">
-        <f>IF(D4&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D4&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K4">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G4,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G4,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L4">
-        <f>SUMPRODUCT((Girdiler!$F$23*D4&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D4-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D4&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D4-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M4">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N4">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D4</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D4</f>
+        <v/>
+      </c>
+      <c r="O4">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D4-G4)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -2010,7 +2117,7 @@
         <v/>
       </c>
       <c r="G5">
-        <f>Girdiler!$F$13*F5</f>
+        <f>Girdiler!$F$16*F5</f>
         <v/>
       </c>
       <c r="H5">
@@ -2018,27 +2125,31 @@
         <v/>
       </c>
       <c r="I5">
-        <f>Girdiler!$F$14*G5*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G5*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J5">
-        <f>IF(D5&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D5&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K5">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G5,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G5,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L5">
-        <f>SUMPRODUCT((Girdiler!$F$23*D5&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D5-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D5&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D5-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M5">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N5">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D5</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D5</f>
+        <v/>
+      </c>
+      <c r="O5">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D5-G5)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -2067,7 +2178,7 @@
         <v/>
       </c>
       <c r="G6">
-        <f>Girdiler!$F$13*F6</f>
+        <f>Girdiler!$F$16*F6</f>
         <v/>
       </c>
       <c r="H6">
@@ -2075,27 +2186,31 @@
         <v/>
       </c>
       <c r="I6">
-        <f>Girdiler!$F$14*G6*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G6*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J6">
-        <f>IF(D6&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D6&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K6">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G6,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G6,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L6">
-        <f>SUMPRODUCT((Girdiler!$F$23*D6&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D6-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D6&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D6-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M6">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N6">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D6</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D6</f>
+        <v/>
+      </c>
+      <c r="O6">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D6-G6)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -2124,7 +2239,7 @@
         <v/>
       </c>
       <c r="G7">
-        <f>Girdiler!$F$13*F7</f>
+        <f>Girdiler!$F$16*F7</f>
         <v/>
       </c>
       <c r="H7">
@@ -2132,27 +2247,31 @@
         <v/>
       </c>
       <c r="I7">
-        <f>Girdiler!$F$14*G7*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G7*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J7">
-        <f>IF(D7&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D7&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K7">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G7,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G7,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L7">
-        <f>SUMPRODUCT((Girdiler!$F$23*D7&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D7-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D7&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D7-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M7">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N7">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D7</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D7</f>
+        <v/>
+      </c>
+      <c r="O7">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D7-G7)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -2181,7 +2300,7 @@
         <v/>
       </c>
       <c r="G8">
-        <f>Girdiler!$F$13*F8</f>
+        <f>Girdiler!$F$16*F8</f>
         <v/>
       </c>
       <c r="H8">
@@ -2189,27 +2308,31 @@
         <v/>
       </c>
       <c r="I8">
-        <f>Girdiler!$F$14*G8*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G8*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J8">
-        <f>IF(D8&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D8&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K8">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G8,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G8,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L8">
-        <f>SUMPRODUCT((Girdiler!$F$23*D8&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D8-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D8&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D8-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M8">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N8">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D8</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D8</f>
+        <v/>
+      </c>
+      <c r="O8">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D8-G8)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -2238,7 +2361,7 @@
         <v/>
       </c>
       <c r="G9">
-        <f>Girdiler!$F$13*F9</f>
+        <f>Girdiler!$F$16*F9</f>
         <v/>
       </c>
       <c r="H9">
@@ -2246,27 +2369,31 @@
         <v/>
       </c>
       <c r="I9">
-        <f>Girdiler!$F$14*G9*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G9*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J9">
-        <f>IF(D9&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D9&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K9">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G9,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G9,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L9">
-        <f>SUMPRODUCT((Girdiler!$F$23*D9&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D9-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D9&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D9-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M9">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N9">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D9</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D9</f>
+        <v/>
+      </c>
+      <c r="O9">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D9-G9)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -2295,7 +2422,7 @@
         <v/>
       </c>
       <c r="G10">
-        <f>Girdiler!$F$13*F10</f>
+        <f>Girdiler!$F$16*F10</f>
         <v/>
       </c>
       <c r="H10">
@@ -2303,27 +2430,31 @@
         <v/>
       </c>
       <c r="I10">
-        <f>Girdiler!$F$14*G10*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G10*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J10">
-        <f>IF(D10&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D10&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K10">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G10,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G10,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L10">
-        <f>SUMPRODUCT((Girdiler!$F$23*D10&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D10-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D10&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D10-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M10">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N10">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D10</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D10</f>
+        <v/>
+      </c>
+      <c r="O10">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D10-G10)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -2352,7 +2483,7 @@
         <v/>
       </c>
       <c r="G11">
-        <f>Girdiler!$F$13*F11</f>
+        <f>Girdiler!$F$16*F11</f>
         <v/>
       </c>
       <c r="H11">
@@ -2360,27 +2491,31 @@
         <v/>
       </c>
       <c r="I11">
-        <f>Girdiler!$F$14*G11*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G11*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J11">
-        <f>IF(D11&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D11&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K11">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G11,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G11,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L11">
-        <f>SUMPRODUCT((Girdiler!$F$23*D11&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D11-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D11&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D11-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M11">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N11">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D11</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D11</f>
+        <v/>
+      </c>
+      <c r="O11">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D11-G11)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -2409,7 +2544,7 @@
         <v/>
       </c>
       <c r="G12">
-        <f>Girdiler!$F$13*F12</f>
+        <f>Girdiler!$F$16*F12</f>
         <v/>
       </c>
       <c r="H12">
@@ -2417,27 +2552,31 @@
         <v/>
       </c>
       <c r="I12">
-        <f>Girdiler!$F$14*G12*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G12*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J12">
-        <f>IF(D12&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D12&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K12">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G12,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G12,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L12">
-        <f>SUMPRODUCT((Girdiler!$F$23*D12&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D12-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D12&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D12-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M12">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N12">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D12</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D12</f>
+        <v/>
+      </c>
+      <c r="O12">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D12-G12)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -2466,7 +2605,7 @@
         <v/>
       </c>
       <c r="G13">
-        <f>Girdiler!$F$13*F13</f>
+        <f>Girdiler!$F$16*F13</f>
         <v/>
       </c>
       <c r="H13">
@@ -2474,27 +2613,31 @@
         <v/>
       </c>
       <c r="I13">
-        <f>Girdiler!$F$14*G13*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G13*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J13">
-        <f>IF(D13&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D13&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K13">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G13,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G13,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L13">
-        <f>SUMPRODUCT((Girdiler!$F$23*D13&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D13-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D13&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D13-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M13">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N13">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D13</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D13</f>
+        <v/>
+      </c>
+      <c r="O13">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D13-G13)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -2523,7 +2666,7 @@
         <v/>
       </c>
       <c r="G14">
-        <f>Girdiler!$F$13*F14</f>
+        <f>Girdiler!$F$16*F14</f>
         <v/>
       </c>
       <c r="H14">
@@ -2531,27 +2674,31 @@
         <v/>
       </c>
       <c r="I14">
-        <f>Girdiler!$F$14*G14*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G14*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J14">
-        <f>IF(D14&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D14&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K14">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G14,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G14,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L14">
-        <f>SUMPRODUCT((Girdiler!$F$23*D14&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D14-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D14&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D14-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M14">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N14">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D14</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D14</f>
+        <v/>
+      </c>
+      <c r="O14">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D14-G14)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -2580,7 +2727,7 @@
         <v/>
       </c>
       <c r="G15">
-        <f>Girdiler!$F$13*F15</f>
+        <f>Girdiler!$F$16*F15</f>
         <v/>
       </c>
       <c r="H15">
@@ -2588,27 +2735,31 @@
         <v/>
       </c>
       <c r="I15">
-        <f>Girdiler!$F$14*G15*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G15*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J15">
-        <f>IF(D15&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D15&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K15">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G15,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G15,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L15">
-        <f>SUMPRODUCT((Girdiler!$F$23*D15&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D15-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D15&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D15-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M15">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N15">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D15</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D15</f>
+        <v/>
+      </c>
+      <c r="O15">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D15-G15)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -2637,7 +2788,7 @@
         <v/>
       </c>
       <c r="G16">
-        <f>Girdiler!$F$13*F16</f>
+        <f>Girdiler!$F$16*F16</f>
         <v/>
       </c>
       <c r="H16">
@@ -2645,27 +2796,31 @@
         <v/>
       </c>
       <c r="I16">
-        <f>Girdiler!$F$14*G16*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G16*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J16">
-        <f>IF(D16&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D16&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K16">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G16,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G16,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L16">
-        <f>SUMPRODUCT((Girdiler!$F$23*D16&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D16-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D16&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D16-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M16">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N16">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D16</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D16</f>
+        <v/>
+      </c>
+      <c r="O16">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D16-G16)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -2694,7 +2849,7 @@
         <v/>
       </c>
       <c r="G17">
-        <f>Girdiler!$F$13*F17</f>
+        <f>Girdiler!$F$16*F17</f>
         <v/>
       </c>
       <c r="H17">
@@ -2702,27 +2857,31 @@
         <v/>
       </c>
       <c r="I17">
-        <f>Girdiler!$F$14*G17*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G17*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J17">
-        <f>IF(D17&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D17&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K17">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G17,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G17,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L17">
-        <f>SUMPRODUCT((Girdiler!$F$23*D17&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D17-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D17&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D17-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M17">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N17">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D17</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D17</f>
+        <v/>
+      </c>
+      <c r="O17">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D17-G17)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -2751,7 +2910,7 @@
         <v/>
       </c>
       <c r="G18">
-        <f>Girdiler!$F$13*F18</f>
+        <f>Girdiler!$F$16*F18</f>
         <v/>
       </c>
       <c r="H18">
@@ -2759,27 +2918,31 @@
         <v/>
       </c>
       <c r="I18">
-        <f>Girdiler!$F$14*G18*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G18*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J18">
-        <f>IF(D18&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D18&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K18">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G18,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G18,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L18">
-        <f>SUMPRODUCT((Girdiler!$F$23*D18&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D18-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D18&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D18-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M18">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N18">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D18</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D18</f>
+        <v/>
+      </c>
+      <c r="O18">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D18-G18)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -2808,7 +2971,7 @@
         <v/>
       </c>
       <c r="G19">
-        <f>Girdiler!$F$13*F19</f>
+        <f>Girdiler!$F$16*F19</f>
         <v/>
       </c>
       <c r="H19">
@@ -2816,27 +2979,31 @@
         <v/>
       </c>
       <c r="I19">
-        <f>Girdiler!$F$14*G19*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G19*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J19">
-        <f>IF(D19&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D19&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K19">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G19,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G19,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L19">
-        <f>SUMPRODUCT((Girdiler!$F$23*D19&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D19-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D19&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D19-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M19">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N19">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D19</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D19</f>
+        <v/>
+      </c>
+      <c r="O19">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D19-G19)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -2865,7 +3032,7 @@
         <v/>
       </c>
       <c r="G20">
-        <f>Girdiler!$F$13*F20</f>
+        <f>Girdiler!$F$16*F20</f>
         <v/>
       </c>
       <c r="H20">
@@ -2873,27 +3040,31 @@
         <v/>
       </c>
       <c r="I20">
-        <f>Girdiler!$F$14*G20*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G20*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J20">
-        <f>IF(D20&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D20&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K20">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G20,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G20,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L20">
-        <f>SUMPRODUCT((Girdiler!$F$23*D20&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D20-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D20&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D20-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M20">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N20">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D20</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D20</f>
+        <v/>
+      </c>
+      <c r="O20">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D20-G20)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -2922,7 +3093,7 @@
         <v/>
       </c>
       <c r="G21">
-        <f>Girdiler!$F$13*F21</f>
+        <f>Girdiler!$F$16*F21</f>
         <v/>
       </c>
       <c r="H21">
@@ -2930,27 +3101,31 @@
         <v/>
       </c>
       <c r="I21">
-        <f>Girdiler!$F$14*G21*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G21*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J21">
-        <f>IF(D21&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D21&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K21">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G21,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G21,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L21">
-        <f>SUMPRODUCT((Girdiler!$F$23*D21&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D21-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D21&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D21-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M21">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N21">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D21</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D21</f>
+        <v/>
+      </c>
+      <c r="O21">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D21-G21)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -2979,7 +3154,7 @@
         <v/>
       </c>
       <c r="G22">
-        <f>Girdiler!$F$13*F22</f>
+        <f>Girdiler!$F$16*F22</f>
         <v/>
       </c>
       <c r="H22">
@@ -2987,27 +3162,31 @@
         <v/>
       </c>
       <c r="I22">
-        <f>Girdiler!$F$14*G22*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G22*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J22">
-        <f>IF(D22&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D22&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K22">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G22,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G22,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L22">
-        <f>SUMPRODUCT((Girdiler!$F$23*D22&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D22-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D22&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D22-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M22">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N22">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D22</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D22</f>
+        <v/>
+      </c>
+      <c r="O22">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D22-G22)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -3036,7 +3215,7 @@
         <v/>
       </c>
       <c r="G23">
-        <f>Girdiler!$F$13*F23</f>
+        <f>Girdiler!$F$16*F23</f>
         <v/>
       </c>
       <c r="H23">
@@ -3044,27 +3223,31 @@
         <v/>
       </c>
       <c r="I23">
-        <f>Girdiler!$F$14*G23*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G23*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J23">
-        <f>IF(D23&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D23&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K23">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G23,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G23,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L23">
-        <f>SUMPRODUCT((Girdiler!$F$23*D23&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D23-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D23&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D23-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M23">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N23">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D23</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D23</f>
+        <v/>
+      </c>
+      <c r="O23">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D23-G23)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -3093,7 +3276,7 @@
         <v/>
       </c>
       <c r="G24">
-        <f>Girdiler!$F$13*F24</f>
+        <f>Girdiler!$F$16*F24</f>
         <v/>
       </c>
       <c r="H24">
@@ -3101,27 +3284,31 @@
         <v/>
       </c>
       <c r="I24">
-        <f>Girdiler!$F$14*G24*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G24*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J24">
-        <f>IF(D24&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D24&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K24">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G24,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G24,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L24">
-        <f>SUMPRODUCT((Girdiler!$F$23*D24&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D24-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D24&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D24-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M24">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N24">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D24</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D24</f>
+        <v/>
+      </c>
+      <c r="O24">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D24-G24)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -3150,7 +3337,7 @@
         <v/>
       </c>
       <c r="G25">
-        <f>Girdiler!$F$13*F25</f>
+        <f>Girdiler!$F$16*F25</f>
         <v/>
       </c>
       <c r="H25">
@@ -3158,27 +3345,31 @@
         <v/>
       </c>
       <c r="I25">
-        <f>Girdiler!$F$14*G25*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G25*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J25">
-        <f>IF(D25&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D25&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K25">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G25,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G25,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L25">
-        <f>SUMPRODUCT((Girdiler!$F$23*D25&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D25-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D25&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D25-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M25">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N25">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D25</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D25</f>
+        <v/>
+      </c>
+      <c r="O25">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D25-G25)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -3207,7 +3398,7 @@
         <v/>
       </c>
       <c r="G26">
-        <f>Girdiler!$F$13*F26</f>
+        <f>Girdiler!$F$16*F26</f>
         <v/>
       </c>
       <c r="H26">
@@ -3215,27 +3406,31 @@
         <v/>
       </c>
       <c r="I26">
-        <f>Girdiler!$F$14*G26*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G26*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J26">
-        <f>IF(D26&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D26&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K26">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G26,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G26,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L26">
-        <f>SUMPRODUCT((Girdiler!$F$23*D26&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D26-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D26&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D26-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M26">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N26">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D26</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D26</f>
+        <v/>
+      </c>
+      <c r="O26">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D26-G26)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -3264,7 +3459,7 @@
         <v/>
       </c>
       <c r="G27">
-        <f>Girdiler!$F$13*F27</f>
+        <f>Girdiler!$F$16*F27</f>
         <v/>
       </c>
       <c r="H27">
@@ -3272,27 +3467,31 @@
         <v/>
       </c>
       <c r="I27">
-        <f>Girdiler!$F$14*G27*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G27*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J27">
-        <f>IF(D27&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D27&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K27">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G27,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G27,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L27">
-        <f>SUMPRODUCT((Girdiler!$F$23*D27&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D27-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D27&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D27-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M27">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N27">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D27</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D27</f>
+        <v/>
+      </c>
+      <c r="O27">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D27-G27)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -3321,7 +3520,7 @@
         <v/>
       </c>
       <c r="G28">
-        <f>Girdiler!$F$13*F28</f>
+        <f>Girdiler!$F$16*F28</f>
         <v/>
       </c>
       <c r="H28">
@@ -3329,27 +3528,31 @@
         <v/>
       </c>
       <c r="I28">
-        <f>Girdiler!$F$14*G28*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G28*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J28">
-        <f>IF(D28&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D28&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K28">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G28,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G28,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L28">
-        <f>SUMPRODUCT((Girdiler!$F$23*D28&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D28-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D28&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D28-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M28">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N28">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D28</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D28</f>
+        <v/>
+      </c>
+      <c r="O28">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D28-G28)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -3378,7 +3581,7 @@
         <v/>
       </c>
       <c r="G29">
-        <f>Girdiler!$F$13*F29</f>
+        <f>Girdiler!$F$16*F29</f>
         <v/>
       </c>
       <c r="H29">
@@ -3386,27 +3589,31 @@
         <v/>
       </c>
       <c r="I29">
-        <f>Girdiler!$F$14*G29*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G29*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J29">
-        <f>IF(D29&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D29&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K29">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G29,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G29,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L29">
-        <f>SUMPRODUCT((Girdiler!$F$23*D29&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D29-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D29&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D29-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M29">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N29">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D29</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D29</f>
+        <v/>
+      </c>
+      <c r="O29">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D29-G29)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -3435,7 +3642,7 @@
         <v/>
       </c>
       <c r="G30">
-        <f>Girdiler!$F$13*F30</f>
+        <f>Girdiler!$F$16*F30</f>
         <v/>
       </c>
       <c r="H30">
@@ -3443,27 +3650,31 @@
         <v/>
       </c>
       <c r="I30">
-        <f>Girdiler!$F$14*G30*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G30*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J30">
-        <f>IF(D30&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D30&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K30">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G30,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G30,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L30">
-        <f>SUMPRODUCT((Girdiler!$F$23*D30&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D30-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D30&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D30-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M30">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N30">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D30</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D30</f>
+        <v/>
+      </c>
+      <c r="O30">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D30-G30)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -3492,7 +3703,7 @@
         <v/>
       </c>
       <c r="G31">
-        <f>Girdiler!$F$13*F31</f>
+        <f>Girdiler!$F$16*F31</f>
         <v/>
       </c>
       <c r="H31">
@@ -3500,27 +3711,31 @@
         <v/>
       </c>
       <c r="I31">
-        <f>Girdiler!$F$14*G31*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G31*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J31">
-        <f>IF(D31&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D31&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K31">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G31,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G31,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L31">
-        <f>SUMPRODUCT((Girdiler!$F$23*D31&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D31-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D31&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D31-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M31">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N31">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D31</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D31</f>
+        <v/>
+      </c>
+      <c r="O31">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D31-G31)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -3549,7 +3764,7 @@
         <v/>
       </c>
       <c r="G32">
-        <f>Girdiler!$F$13*F32</f>
+        <f>Girdiler!$F$16*F32</f>
         <v/>
       </c>
       <c r="H32">
@@ -3557,27 +3772,31 @@
         <v/>
       </c>
       <c r="I32">
-        <f>Girdiler!$F$14*G32*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G32*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J32">
-        <f>IF(D32&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D32&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K32">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G32,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G32,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L32">
-        <f>SUMPRODUCT((Girdiler!$F$23*D32&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D32-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D32&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D32-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M32">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N32">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D32</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D32</f>
+        <v/>
+      </c>
+      <c r="O32">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D32-G32)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -3606,7 +3825,7 @@
         <v/>
       </c>
       <c r="G33">
-        <f>Girdiler!$F$13*F33</f>
+        <f>Girdiler!$F$16*F33</f>
         <v/>
       </c>
       <c r="H33">
@@ -3614,27 +3833,31 @@
         <v/>
       </c>
       <c r="I33">
-        <f>Girdiler!$F$14*G33*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G33*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J33">
-        <f>IF(D33&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D33&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K33">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G33,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G33,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L33">
-        <f>SUMPRODUCT((Girdiler!$F$23*D33&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D33-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D33&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D33-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M33">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N33">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D33</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D33</f>
+        <v/>
+      </c>
+      <c r="O33">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D33-G33)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -3663,7 +3886,7 @@
         <v/>
       </c>
       <c r="G34">
-        <f>Girdiler!$F$13*F34</f>
+        <f>Girdiler!$F$16*F34</f>
         <v/>
       </c>
       <c r="H34">
@@ -3671,27 +3894,31 @@
         <v/>
       </c>
       <c r="I34">
-        <f>Girdiler!$F$14*G34*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G34*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J34">
-        <f>IF(D34&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D34&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K34">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G34,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G34,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L34">
-        <f>SUMPRODUCT((Girdiler!$F$23*D34&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D34-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D34&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D34-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M34">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N34">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D34</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D34</f>
+        <v/>
+      </c>
+      <c r="O34">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D34-G34)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -3720,7 +3947,7 @@
         <v/>
       </c>
       <c r="G35">
-        <f>Girdiler!$F$13*F35</f>
+        <f>Girdiler!$F$16*F35</f>
         <v/>
       </c>
       <c r="H35">
@@ -3728,27 +3955,31 @@
         <v/>
       </c>
       <c r="I35">
-        <f>Girdiler!$F$14*G35*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G35*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J35">
-        <f>IF(D35&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D35&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K35">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G35,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G35,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L35">
-        <f>SUMPRODUCT((Girdiler!$F$23*D35&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D35-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D35&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D35-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M35">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N35">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D35</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D35</f>
+        <v/>
+      </c>
+      <c r="O35">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D35-G35)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -3777,7 +4008,7 @@
         <v/>
       </c>
       <c r="G36">
-        <f>Girdiler!$F$13*F36</f>
+        <f>Girdiler!$F$16*F36</f>
         <v/>
       </c>
       <c r="H36">
@@ -3785,27 +4016,31 @@
         <v/>
       </c>
       <c r="I36">
-        <f>Girdiler!$F$14*G36*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G36*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J36">
-        <f>IF(D36&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D36&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K36">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G36,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G36,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L36">
-        <f>SUMPRODUCT((Girdiler!$F$23*D36&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D36-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D36&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D36-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M36">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N36">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D36</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D36</f>
+        <v/>
+      </c>
+      <c r="O36">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D36-G36)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -3834,7 +4069,7 @@
         <v/>
       </c>
       <c r="G37">
-        <f>Girdiler!$F$13*F37</f>
+        <f>Girdiler!$F$16*F37</f>
         <v/>
       </c>
       <c r="H37">
@@ -3842,27 +4077,31 @@
         <v/>
       </c>
       <c r="I37">
-        <f>Girdiler!$F$14*G37*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G37*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J37">
-        <f>IF(D37&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D37&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K37">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G37,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G37,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L37">
-        <f>SUMPRODUCT((Girdiler!$F$23*D37&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D37-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D37&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D37-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M37">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N37">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D37</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D37</f>
+        <v/>
+      </c>
+      <c r="O37">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D37-G37)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -3891,7 +4130,7 @@
         <v/>
       </c>
       <c r="G38">
-        <f>Girdiler!$F$13*F38</f>
+        <f>Girdiler!$F$16*F38</f>
         <v/>
       </c>
       <c r="H38">
@@ -3899,27 +4138,31 @@
         <v/>
       </c>
       <c r="I38">
-        <f>Girdiler!$F$14*G38*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G38*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J38">
-        <f>IF(D38&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D38&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K38">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G38,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G38,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L38">
-        <f>SUMPRODUCT((Girdiler!$F$23*D38&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D38-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D38&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D38-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M38">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N38">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D38</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D38</f>
+        <v/>
+      </c>
+      <c r="O38">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D38-G38)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -3948,7 +4191,7 @@
         <v/>
       </c>
       <c r="G39">
-        <f>Girdiler!$F$13*F39</f>
+        <f>Girdiler!$F$16*F39</f>
         <v/>
       </c>
       <c r="H39">
@@ -3956,27 +4199,31 @@
         <v/>
       </c>
       <c r="I39">
-        <f>Girdiler!$F$14*G39*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G39*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J39">
-        <f>IF(D39&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D39&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K39">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G39,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G39,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L39">
-        <f>SUMPRODUCT((Girdiler!$F$23*D39&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D39-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D39&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D39-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M39">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N39">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D39</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D39</f>
+        <v/>
+      </c>
+      <c r="O39">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D39-G39)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -4005,7 +4252,7 @@
         <v/>
       </c>
       <c r="G40">
-        <f>Girdiler!$F$13*F40</f>
+        <f>Girdiler!$F$16*F40</f>
         <v/>
       </c>
       <c r="H40">
@@ -4013,27 +4260,31 @@
         <v/>
       </c>
       <c r="I40">
-        <f>Girdiler!$F$14*G40*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G40*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J40">
-        <f>IF(D40&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D40&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K40">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G40,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G40,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L40">
-        <f>SUMPRODUCT((Girdiler!$F$23*D40&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D40-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D40&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D40-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M40">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N40">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D40</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D40</f>
+        <v/>
+      </c>
+      <c r="O40">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D40-G40)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -4062,7 +4313,7 @@
         <v/>
       </c>
       <c r="G41">
-        <f>Girdiler!$F$13*F41</f>
+        <f>Girdiler!$F$16*F41</f>
         <v/>
       </c>
       <c r="H41">
@@ -4070,27 +4321,31 @@
         <v/>
       </c>
       <c r="I41">
-        <f>Girdiler!$F$14*G41*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G41*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J41">
-        <f>IF(D41&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D41&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K41">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G41,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G41,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L41">
-        <f>SUMPRODUCT((Girdiler!$F$23*D41&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D41-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D41&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D41-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M41">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N41">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D41</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D41</f>
+        <v/>
+      </c>
+      <c r="O41">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D41-G41)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -4119,7 +4374,7 @@
         <v/>
       </c>
       <c r="G42">
-        <f>Girdiler!$F$13*F42</f>
+        <f>Girdiler!$F$16*F42</f>
         <v/>
       </c>
       <c r="H42">
@@ -4127,27 +4382,31 @@
         <v/>
       </c>
       <c r="I42">
-        <f>Girdiler!$F$14*G42*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G42*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J42">
-        <f>IF(D42&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D42&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K42">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G42,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G42,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L42">
-        <f>SUMPRODUCT((Girdiler!$F$23*D42&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D42-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D42&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D42-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M42">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N42">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D42</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D42</f>
+        <v/>
+      </c>
+      <c r="O42">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D42-G42)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -4176,7 +4435,7 @@
         <v/>
       </c>
       <c r="G43">
-        <f>Girdiler!$F$13*F43</f>
+        <f>Girdiler!$F$16*F43</f>
         <v/>
       </c>
       <c r="H43">
@@ -4184,27 +4443,31 @@
         <v/>
       </c>
       <c r="I43">
-        <f>Girdiler!$F$14*G43*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G43*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J43">
-        <f>IF(D43&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D43&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K43">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G43,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G43,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L43">
-        <f>SUMPRODUCT((Girdiler!$F$23*D43&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D43-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D43&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D43-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M43">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N43">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D43</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D43</f>
+        <v/>
+      </c>
+      <c r="O43">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D43-G43)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -4233,7 +4496,7 @@
         <v/>
       </c>
       <c r="G44">
-        <f>Girdiler!$F$13*F44</f>
+        <f>Girdiler!$F$16*F44</f>
         <v/>
       </c>
       <c r="H44">
@@ -4241,27 +4504,31 @@
         <v/>
       </c>
       <c r="I44">
-        <f>Girdiler!$F$14*G44*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G44*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J44">
-        <f>IF(D44&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D44&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K44">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G44,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G44,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L44">
-        <f>SUMPRODUCT((Girdiler!$F$23*D44&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D44-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D44&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D44-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M44">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N44">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D44</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D44</f>
+        <v/>
+      </c>
+      <c r="O44">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D44-G44)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -4290,7 +4557,7 @@
         <v/>
       </c>
       <c r="G45">
-        <f>Girdiler!$F$13*F45</f>
+        <f>Girdiler!$F$16*F45</f>
         <v/>
       </c>
       <c r="H45">
@@ -4298,27 +4565,31 @@
         <v/>
       </c>
       <c r="I45">
-        <f>Girdiler!$F$14*G45*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G45*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J45">
-        <f>IF(D45&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D45&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K45">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G45,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G45,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L45">
-        <f>SUMPRODUCT((Girdiler!$F$23*D45&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D45-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D45&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D45-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M45">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N45">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D45</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D45</f>
+        <v/>
+      </c>
+      <c r="O45">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D45-G45)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -4347,7 +4618,7 @@
         <v/>
       </c>
       <c r="G46">
-        <f>Girdiler!$F$13*F46</f>
+        <f>Girdiler!$F$16*F46</f>
         <v/>
       </c>
       <c r="H46">
@@ -4355,27 +4626,31 @@
         <v/>
       </c>
       <c r="I46">
-        <f>Girdiler!$F$14*G46*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G46*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J46">
-        <f>IF(D46&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D46&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K46">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G46,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G46,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L46">
-        <f>SUMPRODUCT((Girdiler!$F$23*D46&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D46-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D46&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D46-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M46">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N46">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D46</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D46</f>
+        <v/>
+      </c>
+      <c r="O46">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D46-G46)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -4404,7 +4679,7 @@
         <v/>
       </c>
       <c r="G47">
-        <f>Girdiler!$F$13*F47</f>
+        <f>Girdiler!$F$16*F47</f>
         <v/>
       </c>
       <c r="H47">
@@ -4412,27 +4687,31 @@
         <v/>
       </c>
       <c r="I47">
-        <f>Girdiler!$F$14*G47*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G47*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J47">
-        <f>IF(D47&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D47&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K47">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G47,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G47,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L47">
-        <f>SUMPRODUCT((Girdiler!$F$23*D47&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D47-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D47&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D47-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M47">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N47">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D47</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D47</f>
+        <v/>
+      </c>
+      <c r="O47">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D47-G47)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -4461,7 +4740,7 @@
         <v/>
       </c>
       <c r="G48">
-        <f>Girdiler!$F$13*F48</f>
+        <f>Girdiler!$F$16*F48</f>
         <v/>
       </c>
       <c r="H48">
@@ -4469,27 +4748,31 @@
         <v/>
       </c>
       <c r="I48">
-        <f>Girdiler!$F$14*G48*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G48*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J48">
-        <f>IF(D48&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D48&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K48">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G48,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G48,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L48">
-        <f>SUMPRODUCT((Girdiler!$F$23*D48&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D48-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D48&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D48-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M48">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N48">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D48</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D48</f>
+        <v/>
+      </c>
+      <c r="O48">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D48-G48)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -4518,7 +4801,7 @@
         <v/>
       </c>
       <c r="G49">
-        <f>Girdiler!$F$13*F49</f>
+        <f>Girdiler!$F$16*F49</f>
         <v/>
       </c>
       <c r="H49">
@@ -4526,27 +4809,31 @@
         <v/>
       </c>
       <c r="I49">
-        <f>Girdiler!$F$14*G49*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G49*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J49">
-        <f>IF(D49&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D49&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K49">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G49,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G49,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L49">
-        <f>SUMPRODUCT((Girdiler!$F$23*D49&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D49-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D49&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D49-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M49">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N49">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D49</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D49</f>
+        <v/>
+      </c>
+      <c r="O49">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D49-G49)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -4575,7 +4862,7 @@
         <v/>
       </c>
       <c r="G50">
-        <f>Girdiler!$F$13*F50</f>
+        <f>Girdiler!$F$16*F50</f>
         <v/>
       </c>
       <c r="H50">
@@ -4583,27 +4870,31 @@
         <v/>
       </c>
       <c r="I50">
-        <f>Girdiler!$F$14*G50*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G50*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J50">
-        <f>IF(D50&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D50&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K50">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G50,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G50,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L50">
-        <f>SUMPRODUCT((Girdiler!$F$23*D50&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D50-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D50&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D50-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M50">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N50">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D50</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D50</f>
+        <v/>
+      </c>
+      <c r="O50">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D50-G50)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -4632,7 +4923,7 @@
         <v/>
       </c>
       <c r="G51">
-        <f>Girdiler!$F$13*F51</f>
+        <f>Girdiler!$F$16*F51</f>
         <v/>
       </c>
       <c r="H51">
@@ -4640,27 +4931,31 @@
         <v/>
       </c>
       <c r="I51">
-        <f>Girdiler!$F$14*G51*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G51*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J51">
-        <f>IF(D51&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D51&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K51">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G51,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G51,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L51">
-        <f>SUMPRODUCT((Girdiler!$F$23*D51&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D51-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D51&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D51-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M51">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N51">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D51</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D51</f>
+        <v/>
+      </c>
+      <c r="O51">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D51-G51)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -4689,7 +4984,7 @@
         <v/>
       </c>
       <c r="G52">
-        <f>Girdiler!$F$13*F52</f>
+        <f>Girdiler!$F$16*F52</f>
         <v/>
       </c>
       <c r="H52">
@@ -4697,27 +4992,31 @@
         <v/>
       </c>
       <c r="I52">
-        <f>Girdiler!$F$14*G52*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G52*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J52">
-        <f>IF(D52&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D52&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K52">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G52,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G52,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L52">
-        <f>SUMPRODUCT((Girdiler!$F$23*D52&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D52-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D52&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D52-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M52">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N52">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D52</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D52</f>
+        <v/>
+      </c>
+      <c r="O52">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D52-G52)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -4746,7 +5045,7 @@
         <v/>
       </c>
       <c r="G53">
-        <f>Girdiler!$F$13*F53</f>
+        <f>Girdiler!$F$16*F53</f>
         <v/>
       </c>
       <c r="H53">
@@ -4754,27 +5053,31 @@
         <v/>
       </c>
       <c r="I53">
-        <f>Girdiler!$F$14*G53*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G53*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J53">
-        <f>IF(D53&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D53&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K53">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G53,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G53,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L53">
-        <f>SUMPRODUCT((Girdiler!$F$23*D53&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D53-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D53&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D53-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M53">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N53">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D53</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D53</f>
+        <v/>
+      </c>
+      <c r="O53">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D53-G53)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -4803,7 +5106,7 @@
         <v/>
       </c>
       <c r="G54">
-        <f>Girdiler!$F$13*F54</f>
+        <f>Girdiler!$F$16*F54</f>
         <v/>
       </c>
       <c r="H54">
@@ -4811,27 +5114,31 @@
         <v/>
       </c>
       <c r="I54">
-        <f>Girdiler!$F$14*G54*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G54*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J54">
-        <f>IF(D54&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D54&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K54">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G54,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G54,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L54">
-        <f>SUMPRODUCT((Girdiler!$F$23*D54&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D54-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D54&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D54-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M54">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N54">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D54</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D54</f>
+        <v/>
+      </c>
+      <c r="O54">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D54-G54)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -4860,7 +5167,7 @@
         <v/>
       </c>
       <c r="G55">
-        <f>Girdiler!$F$13*F55</f>
+        <f>Girdiler!$F$16*F55</f>
         <v/>
       </c>
       <c r="H55">
@@ -4868,27 +5175,31 @@
         <v/>
       </c>
       <c r="I55">
-        <f>Girdiler!$F$14*G55*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G55*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J55">
-        <f>IF(D55&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D55&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K55">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G55,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G55,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L55">
-        <f>SUMPRODUCT((Girdiler!$F$23*D55&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D55-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D55&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D55-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M55">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N55">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D55</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D55</f>
+        <v/>
+      </c>
+      <c r="O55">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D55-G55)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -4917,7 +5228,7 @@
         <v/>
       </c>
       <c r="G56">
-        <f>Girdiler!$F$13*F56</f>
+        <f>Girdiler!$F$16*F56</f>
         <v/>
       </c>
       <c r="H56">
@@ -4925,27 +5236,31 @@
         <v/>
       </c>
       <c r="I56">
-        <f>Girdiler!$F$14*G56*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G56*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J56">
-        <f>IF(D56&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D56&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K56">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G56,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G56,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L56">
-        <f>SUMPRODUCT((Girdiler!$F$23*D56&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D56-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D56&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D56-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M56">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N56">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D56</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D56</f>
+        <v/>
+      </c>
+      <c r="O56">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D56-G56)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -4974,7 +5289,7 @@
         <v/>
       </c>
       <c r="G57">
-        <f>Girdiler!$F$13*F57</f>
+        <f>Girdiler!$F$16*F57</f>
         <v/>
       </c>
       <c r="H57">
@@ -4982,27 +5297,31 @@
         <v/>
       </c>
       <c r="I57">
-        <f>Girdiler!$F$14*G57*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G57*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J57">
-        <f>IF(D57&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D57&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K57">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G57,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G57,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L57">
-        <f>SUMPRODUCT((Girdiler!$F$23*D57&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D57-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D57&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D57-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M57">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N57">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D57</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D57</f>
+        <v/>
+      </c>
+      <c r="O57">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D57-G57)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -5031,7 +5350,7 @@
         <v/>
       </c>
       <c r="G58">
-        <f>Girdiler!$F$13*F58</f>
+        <f>Girdiler!$F$16*F58</f>
         <v/>
       </c>
       <c r="H58">
@@ -5039,27 +5358,31 @@
         <v/>
       </c>
       <c r="I58">
-        <f>Girdiler!$F$14*G58*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G58*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J58">
-        <f>IF(D58&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D58&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K58">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G58,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G58,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L58">
-        <f>SUMPRODUCT((Girdiler!$F$23*D58&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D58-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D58&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D58-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M58">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N58">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D58</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D58</f>
+        <v/>
+      </c>
+      <c r="O58">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D58-G58)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -5088,7 +5411,7 @@
         <v/>
       </c>
       <c r="G59">
-        <f>Girdiler!$F$13*F59</f>
+        <f>Girdiler!$F$16*F59</f>
         <v/>
       </c>
       <c r="H59">
@@ -5096,27 +5419,31 @@
         <v/>
       </c>
       <c r="I59">
-        <f>Girdiler!$F$14*G59*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G59*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J59">
-        <f>IF(D59&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D59&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K59">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G59,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G59,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L59">
-        <f>SUMPRODUCT((Girdiler!$F$23*D59&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D59-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D59&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D59-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M59">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N59">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D59</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D59</f>
+        <v/>
+      </c>
+      <c r="O59">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D59-G59)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -5145,7 +5472,7 @@
         <v/>
       </c>
       <c r="G60">
-        <f>Girdiler!$F$13*F60</f>
+        <f>Girdiler!$F$16*F60</f>
         <v/>
       </c>
       <c r="H60">
@@ -5153,27 +5480,31 @@
         <v/>
       </c>
       <c r="I60">
-        <f>Girdiler!$F$14*G60*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G60*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J60">
-        <f>IF(D60&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D60&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K60">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G60,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G60,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L60">
-        <f>SUMPRODUCT((Girdiler!$F$23*D60&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D60-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D60&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D60-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M60">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N60">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D60</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D60</f>
+        <v/>
+      </c>
+      <c r="O60">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D60-G60)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -5202,7 +5533,7 @@
         <v/>
       </c>
       <c r="G61">
-        <f>Girdiler!$F$13*F61</f>
+        <f>Girdiler!$F$16*F61</f>
         <v/>
       </c>
       <c r="H61">
@@ -5210,27 +5541,31 @@
         <v/>
       </c>
       <c r="I61">
-        <f>Girdiler!$F$14*G61*(1-Girdiler!$F$16)*(1+Girdiler!$F$15)</f>
+        <f>Girdiler!$F$17*G61*(1-Girdiler!$F$19)*(1+Girdiler!$F$18)</f>
         <v/>
       </c>
       <c r="J61">
-        <f>IF(D61&gt;=12*Girdiler!$F$6,Girdiler!$F$19*Girdiler!$F$18*Girdiler!$F$6*Girdiler!$F$17,0)</f>
+        <f>IF(D61&gt;=12*Girdiler!$F$6,Girdiler!$F$22*Girdiler!$F$21*Girdiler!$F$6*Girdiler!$F$20,0)</f>
         <v/>
       </c>
       <c r="K61">
-        <f>Girdiler!$F$20*MIN(Girdiler!$F$22*G61,Girdiler!$F$21)</f>
+        <f>Girdiler!$F$23*MIN(Girdiler!$F$25*G61,Girdiler!$F$24)</f>
         <v/>
       </c>
       <c r="L61">
-        <f>SUMPRODUCT((Girdiler!$F$23*D61&gt;Girdiler!$D$47:$D$51)*(Girdiler!$F$23*D61-Girdiler!$D$47:$D$51)*Girdiler!$C$47:$C$51)</f>
+        <f>SUMPRODUCT((Girdiler!$F$26*D61&gt;Girdiler!$D$50:$D$54)*(Girdiler!$F$26*D61-Girdiler!$D$50:$D$54)*Girdiler!$C$50:$C$54)</f>
         <v/>
       </c>
       <c r="M61">
-        <f>Girdiler!$F$25*Girdiler!$F$24*(1-Girdiler!$F$11)</f>
+        <f>Girdiler!$F$28*Girdiler!$F$27*(1-Girdiler!$F$14)</f>
         <v/>
       </c>
       <c r="N61">
-        <f>Girdiler!$F$27*Girdiler!$F$26*Girdiler!$F$23*D61</f>
+        <f>Girdiler!$F$30*Girdiler!$F$29*Girdiler!$F$26*D61</f>
+        <v/>
+      </c>
+      <c r="O61">
+        <f>12*Girdiler!$F$12*Girdiler!$F$13*MIN(MAX(((D61-G61)/12-Girdiler!$F$6/3)/(Girdiler!$F$11*Girdiler!$F$6-Girdiler!$F$6/3),0),1)</f>
         <v/>
       </c>
     </row>
@@ -5245,7 +5580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -5354,7 +5689,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>B5*(Girdiler!$F$10*SUMPRODUCT(Hesap!$E$2:$E$61,Hesap!$L$2:$L$61)+Girdiler!$F$12*SUMPRODUCT(Hesap!$E$2:$E$61,Hesap!$N$2:$N$61))</f>
+        <f>B5*(Girdiler!$F$10*SUMPRODUCT(Hesap!$E$2:$E$61,Hesap!$L$2:$L$61)+Girdiler!$F$15*SUMPRODUCT(Hesap!$E$2:$E$61,Hesap!$N$2:$N$61))</f>
         <v/>
       </c>
     </row>
@@ -5376,7 +5711,7 @@
         </is>
       </c>
       <c r="B12">
-        <f>MAX(Girdiler!$F$30*(1-Girdiler!$F$31)*Girdiler!$F$28*B5*B2*(Girdiler!$F$29-B4),0)</f>
+        <f>MAX(Girdiler!$F$33*(1-Girdiler!$F$34)*Girdiler!$F$31*B5*B2*(Girdiler!$F$32-B4),0)</f>
         <v/>
       </c>
     </row>
@@ -5387,7 +5722,7 @@
         </is>
       </c>
       <c r="B13">
-        <f>B5*Girdiler!$F$32*Girdiler!$F$35*B2*Girdiler!$F$33*(1-Girdiler!$F$34)</f>
+        <f>B5*Girdiler!$F$35*Girdiler!$F$38*B2*Girdiler!$F$36*(1-Girdiler!$F$37)</f>
         <v/>
       </c>
     </row>
@@ -5398,7 +5733,7 @@
         </is>
       </c>
       <c r="B14">
-        <f>Girdiler!$F$39</f>
+        <f>Girdiler!$F$42</f>
         <v/>
       </c>
     </row>
@@ -5409,7 +5744,7 @@
         </is>
       </c>
       <c r="B15">
-        <f>B5*Girdiler!$F$40*Girdiler!$F$41</f>
+        <f>B5*Girdiler!$F$43*Girdiler!$F$44</f>
         <v/>
       </c>
     </row>
@@ -5420,36 +5755,47 @@
         </is>
       </c>
       <c r="B16">
-        <f>Girdiler!$F$42*B6</f>
+        <f>Girdiler!$F$45*B6</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Gelire bağlı yeni prim (TL)</t>
+        </is>
+      </c>
+      <c r="B17">
+        <f>B5*(1-Girdiler!$F$15)*SUMPRODUCT(Hesap!$E$2:$E$61,Hesap!$O$2:$O$61)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>NET HAZİNE ETKİSİ (TL/yıl)</t>
         </is>
       </c>
-      <c r="B17" s="4">
-        <f>B6-B7-B8-B9-B10-B11-B12-B13-B14-B15-B16</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="B18" s="4">
+        <f>B6+B17-B7-B8-B9-B10-B11-B12-B13-B14-B15-B16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>Net (milyar TL)</t>
         </is>
       </c>
-      <c r="B18">
-        <f>B17/1000000000</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Not: prim_devam=0 en kötü hâldir (eski kayıtlıların primi hiç sürmez); varyantlar Senaryolar_Python sayfasındadır.</t>
+      <c r="B19">
+        <f>B18/1000000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Not: eski sabit prim kalktı; yerine gelire bağlı prim (Girdiler: prim_k, prim_ay); varyantlar Senaryolar_Python sayfasındadır.</t>
         </is>
       </c>
     </row>
@@ -5464,7 +5810,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C49"/>
+  <dimension ref="A1:C51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -5501,10 +5847,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-2.013885121244206</v>
+        <v>-2.048110252063701</v>
       </c>
       <c r="C4" t="n">
-        <v>-6.41445985704332</v>
+        <v>-6.518307808347563</v>
       </c>
     </row>
     <row r="5">
@@ -5514,10 +5860,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1.318681980023</v>
+        <v>1.6413105825489</v>
       </c>
       <c r="C5" t="n">
-        <v>3.69521576662539</v>
+        <v>4.674154885402459</v>
       </c>
     </row>
     <row r="6">
@@ -5527,10 +5873,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>23.71682554050645</v>
+        <v>26.56432895445933</v>
       </c>
       <c r="C6" t="n">
-        <v>71.64972496970631</v>
+        <v>80.28979116639738</v>
       </c>
     </row>
     <row r="8">
@@ -5543,41 +5889,41 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>V0 Baz: %13,5; eski kayıtlıların primi hiç sürmez</t>
+          <t>V0 Baz: %13,5; gelire bağlı prim, tam prim 6 asgari ücrette</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1.318681980023</v>
+        <v>1.6413105825489</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>V1 Eski kayıtlıların %50'si primi sürdürür</t>
+          <t>V1 Gelire bağlı prim hiç alınmasaydı (prim sıfır)</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4.132824120023001</v>
+        <v>0.3955031889298513</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>V2 %75'i sürdürür</t>
+          <t>V2 Tam prim eşiği 3 asgari ücret</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>5.539895190023</v>
+        <v>3.042843900370332</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>V3 Hepsi sürdürür</t>
+          <t>V3 Tam prim eşiği 12 asgari ücret</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6.946966260023002</v>
+        <v>1.000609637259104</v>
       </c>
     </row>
     <row r="13">
@@ -5587,7 +5933,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>5.605830913815579</v>
+        <v>5.752387877450135</v>
       </c>
     </row>
     <row r="14">
@@ -5597,17 +5943,17 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>10.23467206349843</v>
+        <v>10.19932119480739</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>V7 Ücretli çalışana izin verilseydi (u=%20)</t>
+          <t>V7 Maaşlı hiç mikro mükellef olmasaydı (u=0)</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.3955031889298513</v>
+        <v>2.875941222046813</v>
       </c>
     </row>
     <row r="16">
@@ -5617,17 +5963,17 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>3.429288585022999</v>
+        <v>3.7519171875489</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>V9 SGK tahsil oranı %100</t>
+          <t>V9 Gelire bağlı primin tahsil oranı %80</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>-0.08838908997700055</v>
+        <v>1.39214910382509</v>
       </c>
     </row>
     <row r="18">
@@ -5637,7 +5983,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>-35.08074749647865</v>
+        <v>-34.75811889395275</v>
       </c>
     </row>
     <row r="19">
@@ -5647,7 +5993,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1.658587936400376</v>
+        <v>1.981216538926277</v>
       </c>
     </row>
     <row r="20">
@@ -5657,7 +6003,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1.936435777712903</v>
+        <v>2.259064380238804</v>
       </c>
     </row>
     <row r="22">
@@ -5667,7 +6013,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.1807938805398902</v>
+        <v>0.1883279083005191</v>
       </c>
     </row>
     <row r="24">
@@ -5684,7 +6030,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>-6.355437545210761</v>
+        <v>-16.34800279896533</v>
       </c>
     </row>
     <row r="26">
@@ -5694,7 +6040,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>-3.380972462056701</v>
+        <v>-10.95323132106929</v>
       </c>
     </row>
     <row r="27">
@@ -5704,7 +6050,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>0.3984784252397677</v>
+        <v>-4.96310105473143</v>
       </c>
     </row>
     <row r="28">
@@ -5714,7 +6060,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>2.93701569013757</v>
+        <v>-0.4736696384264011</v>
       </c>
     </row>
     <row r="29">
@@ -5724,7 +6070,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>5.812795204092121</v>
+        <v>2.745564477485866</v>
       </c>
     </row>
     <row r="30">
@@ -5734,7 +6080,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>9.342409413022768</v>
+        <v>6.168665916403549</v>
       </c>
     </row>
     <row r="31">
@@ -5744,7 +6090,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>12.12628166050324</v>
+        <v>8.553404119724528</v>
       </c>
     </row>
     <row r="32">
@@ -5754,7 +6100,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>0.77025</v>
+        <v>0.4645</v>
       </c>
     </row>
     <row r="34">
@@ -5771,10 +6117,10 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>-1.964913826520587</v>
+        <v>-1.88238452487336</v>
       </c>
       <c r="C35" t="n">
-        <v>8.915990083475434</v>
+        <v>8.558010612258492</v>
       </c>
     </row>
     <row r="36">
@@ -5793,27 +6139,27 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>prim_devam</t>
+          <t>n_toplam</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>0</v>
+        <v>-1.180340618032616</v>
       </c>
       <c r="C37" t="n">
-        <v>5.628284280000002</v>
+        <v>3.908920228549581</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>n_toplam</t>
+          <t>medyan_W</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>-0.9551828924027577</v>
+        <v>-2.726409764881736</v>
       </c>
       <c r="C38" t="n">
-        <v>3.163268020294853</v>
+        <v>2.968999848105354</v>
       </c>
     </row>
     <row r="39">
@@ -5826,136 +6172,162 @@
         <v>2.814142140000001</v>
       </c>
       <c r="C39" t="n">
-        <v>-1.40707107</v>
+        <v>-1.407071070000001</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>medyan_W</t>
+          <t>prim_k</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>-2.372042154910663</v>
+        <v>1.401533317821432</v>
       </c>
       <c r="C40" t="n">
-        <v>2.463885342496412</v>
+        <v>-0.6407009452897967</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>sigma</t>
+          <t>u_ucretli</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>-0.3384366074561423</v>
+        <v>1.234630639497912</v>
       </c>
       <c r="C41" t="n">
-        <v>-0.1350771362789137</v>
+        <v>-1.234630639497911</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>kdv_donanim_pay</t>
+          <t>prim_toplama</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>0.3088768988449516</v>
+        <v>-0.6229036968095244</v>
       </c>
       <c r="C42" t="n">
-        <v>-0.3088768988449515</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>marj</t>
+          <t>sigma</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>0.2516794350287991</v>
+        <v>-0.6019303148476094</v>
       </c>
       <c r="C43" t="n">
-        <v>-0.2702672355060652</v>
+        <v>-0.03328261409559465</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>myo_uygun</t>
+          <t>marj</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>0.2427899688409824</v>
+        <v>0.5286330723567436</v>
       </c>
       <c r="C44" t="n">
-        <v>-0.2427899688409824</v>
+        <v>-0.5472208728340101</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>kgf_alim</t>
+          <t>kdv_donanim_pay</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>0.07180279486280036</v>
+        <v>0.3088768988449516</v>
       </c>
       <c r="C45" t="n">
-        <v>-0.1196713247713342</v>
+        <v>-0.3088768988449516</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>kgf_temerrut</t>
+          <t>myo_uygun</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>0.05983566238566685</v>
+        <v>0.2427899688409824</v>
       </c>
       <c r="C46" t="n">
-        <v>-0.1196713247713342</v>
+        <v>-0.2427899688409824</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>bes_vazgecme</t>
+          <t>kgf_alim</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>-0.08308609119838332</v>
+        <v>0.07180279486280036</v>
       </c>
       <c r="C47" t="n">
-        <v>0.08308609119838332</v>
+        <v>-0.1196713247713342</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>phi</t>
+          <t>kgf_temerrut</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>0.02752440469740677</v>
+        <v>0.05983566238566685</v>
       </c>
       <c r="C48" t="n">
-        <v>-0.05504880939481378</v>
+        <v>-0.1196713247713342</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
+          <t>bes_vazgecme</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>-0.08308609119838332</v>
+      </c>
+      <c r="C49" t="n">
+        <v>0.08308609119838332</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>phi</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>0.02752440469740677</v>
+      </c>
+      <c r="C50" t="n">
+        <v>-0.05504880939481378</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
           <t>onlem</t>
         </is>
       </c>
-      <c r="B49" t="n">
+      <c r="B51" t="n">
         <v>-0.01651464281844425</v>
       </c>
-      <c r="C49" t="n">
+      <c r="C51" t="n">
         <v>0.01651464281844401</v>
       </c>
     </row>

</xml_diff>